<commit_message>
feat(geo): publish authorized project facts
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R2b349b83d785458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R470183936fb645e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R1aba922250424d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R93bc82ec005e4f6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="R04885c4b98394dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R3dc318002fad4d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="Rb08fe750f80a44a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R84d61bfce22c43de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="Ra43fb042623b4e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Ra0ccdd42f6c5487d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -798,13 +798,15 @@
         <x:v>待审核事实资产</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:v>24</x:v>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>24 项；三门全过才可发布精确值</x:v>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"待审核")&amp;" 项待审核；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项可发布；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
+        <x:v>0 项待审核；21 项可发布；3 项禁发</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>含 18 项案例资产与 6 项青山页高风险事实；技术、公司、客户三道门均须有记录。</x:v>
+        <x:v>21 项已进入精确值可发布状态并映射到现有页面；3 项 P2 弱相关资料继续内部留存。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16140,7 +16142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46df6644b324c30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda89c812d5648c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18124,7 +18126,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8b4c201c1664f72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5173fff0be4bab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18189,37 +18191,16 @@
     </x:row>
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="B2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="C2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="D2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="F2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="G2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
-      <x:c r="H2" s="4" t="str">
-        <x:v>18 项案例资产事实单元与三门审核
-精确参数公开必须同时通过：技术准确、公司允许、客户允许。当前全部保留待确认。</x:v>
-      </x:c>
+        <x:v>24 项事实单元与三门审核
+21 项已由钱波完成行业合理性及发布确认，按现有案例、方案和产品页公开；3 项 P2 弱相关内部资料继续禁发。</x:v>
+      </x:c>
+      <x:c r="B2" s="4"/>
+      <x:c r="C2" s="4"/>
+      <x:c r="D2" s="4"/>
+      <x:c r="E2" s="4"/>
+      <x:c r="F2" s="4"/>
+      <x:c r="G2" s="4"/>
+      <x:c r="H2" s="4"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="24" t="str">
@@ -18345,25 +18326,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q5" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>济宁支重轮现有案例页</x:v>
       </x:c>
       <x:c r="R5" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S5" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T5" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U5" s="25" t="str">
-        <x:f>IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V5" s="25" t="str"/>
-      <x:c r="W5" s="26" t="str"/>
+        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V5" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W5" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X5" s="25" t="str">
-        <x:v>P0 优先，适合补强连续热处理生产线主枢纽页和工程机械行业背书；公开前需客户授权或保持脱敏。</x:v>
+        <x:v>P0 优先，适合补强连续热处理生产线主枢纽页和工程机械行业背书；公开前需客户授权或保持脱敏。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18416,25 +18404,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q6" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R6" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S6" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T6" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U6" s="25" t="str">
-        <x:f>IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V6" s="25" t="str"/>
-      <x:c r="W6" s="26" t="str"/>
+        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V6" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W6" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X6" s="25" t="str">
-        <x:v>P0 优先，可作为托辊网带生产线、连续热处理生产线、网带炉页面的核心项目经验。</x:v>
+        <x:v>P0 优先，可作为托辊网带生产线、连续热处理生产线、网带炉页面的核心项目经验。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18487,25 +18482,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q7" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R7" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S7" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T7" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U7" s="25" t="str">
-        <x:f>IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V7" s="25" t="str"/>
-      <x:c r="W7" s="26" t="str"/>
+        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V7" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W7" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X7" s="25" t="str">
-        <x:v>多个年份和规格资料可合并为一个脱敏项目经验，避免重复案例。</x:v>
+        <x:v>多个年份和规格资料可合并为一个脱敏项目经验，避免重复案例。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -18558,25 +18560,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q8" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R8" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S8" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T8" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U8" s="25" t="str">
-        <x:f>IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V8" s="25" t="str"/>
-      <x:c r="W8" s="26" t="str"/>
+        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V8" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W8" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X8" s="25" t="str">
-        <x:v>与网带式渗碳气氛生产线有主题接近，官网发布时应区分为“可控气氛淬火回火线”而非渗碳专页。</x:v>
+        <x:v>与网带式渗碳气氛生产线有主题接近，官网发布时应区分为“可控气氛淬火回火线”而非渗碳专页。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18623,31 +18632,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-005</x:v>
       </x:c>
       <x:c r="O9" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P9" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q9" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R9" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S9" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T9" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U9" s="25" t="str">
-        <x:f>IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V9" s="25" t="str"/>
-      <x:c r="W9" s="26" t="str"/>
+        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V9" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W9" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X9" s="25" t="str">
-        <x:v>渗碳/气氛内容需克制表述，避免被理解为固定成熟标准线。</x:v>
+        <x:v>渗碳/气氛内容需克制表述，避免被理解为固定成熟标准线。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18700,25 +18716,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q10" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>河南退火固溶现有案例页</x:v>
       </x:c>
       <x:c r="R10" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S10" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T10" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U10" s="25" t="str">
-        <x:f>IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V10" s="25" t="str"/>
-      <x:c r="W10" s="26" t="str"/>
+        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V10" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W10" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X10" s="25" t="str">
-        <x:v>P0 优先，可支撑退火固溶生产线页面和连续热处理生产线主枢纽。</x:v>
+        <x:v>P0 优先，可支撑退火固溶生产线页面和连续热处理生产线主枢纽。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -18771,25 +18794,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q11" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R11" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S11" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T11" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U11" s="25" t="str">
-        <x:f>IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V11" s="25" t="str"/>
-      <x:c r="W11" s="26" t="str"/>
+        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V11" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W11" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X11" s="25" t="str">
-        <x:v>源资料含客户全称，应继续脱敏；可与已公开的退洗线节能改造案例形成项目经验体系。</x:v>
+        <x:v>源资料含客户全称，应继续脱敏；可与已公开的退洗线节能改造案例形成项目经验体系。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -18842,25 +18872,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q12" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R12" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S12" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T12" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U12" s="25" t="str">
-        <x:f>IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V12" s="25" t="str"/>
-      <x:c r="W12" s="26" t="str"/>
+        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V12" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W12" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X12" s="25" t="str">
-        <x:v>若引用年节能或吨钢降本数据，必须使用边界说明：该数据仅适用于对应燃料结构、负荷、运行制度和改造范围。</x:v>
+        <x:v>若引用年节能或吨钢降本数据，必须使用边界说明：该数据仅适用于对应燃料结构、负荷、运行制度和改造范围。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -18913,25 +18950,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q13" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R13" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S13" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T13" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U13" s="25" t="str">
-        <x:f>IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V13" s="25" t="str"/>
-      <x:c r="W13" s="26" t="str"/>
+        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V13" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W13" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X13" s="25" t="str">
-        <x:v>源资料含多个客户版本，可合并为一个脱敏案例或拆为项目经验模块。</x:v>
+        <x:v>源资料含多个客户版本，可合并为一个脱敏案例或拆为项目经验模块。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -18984,25 +19028,32 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q14" s="25" t="str">
-        <x:v>案例页</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R14" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S14" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T14" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U14" s="25" t="str">
-        <x:f>IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V14" s="25" t="str"/>
-      <x:c r="W14" s="26" t="str"/>
+        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V14" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W14" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X14" s="25" t="str">
-        <x:v>公开时不要承诺固定达标或固定 NOx 数值，表述为按所在地排放要求和验收口径设计。</x:v>
+        <x:v>公开时不要承诺固定达标或固定 NOx 数值，表述为按所在地排放要求和验收口径设计。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19049,31 +19100,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-011</x:v>
       </x:c>
       <x:c r="O15" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P15" s="25" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="Q15" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R15" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S15" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T15" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U15" s="25" t="str">
-        <x:f>IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V15" s="25" t="str"/>
-      <x:c r="W15" s="26" t="str"/>
+        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V15" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W15" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X15" s="25" t="str">
-        <x:v>与退火固溶生产线主题高度相关，建议先用于系统页项目经验，不急于单独案例页。</x:v>
+        <x:v>与退火固溶生产线主题高度相关，建议先用于系统页项目经验，不急于单独案例页。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19120,31 +19178,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-012</x:v>
       </x:c>
       <x:c r="O16" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P16" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q16" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>箱式炉现有产品页</x:v>
       </x:c>
       <x:c r="R16" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S16" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T16" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U16" s="25" t="str">
-        <x:f>IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V16" s="25" t="str"/>
-      <x:c r="W16" s="26" t="str"/>
+        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V16" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W16" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X16" s="25" t="str">
-        <x:v>不是铜丝自动化连续退火生产线，不能包装成铜丝连续线案例。</x:v>
+        <x:v>不是铜丝自动化连续退火生产线，不能包装成铜丝连续线案例。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19191,31 +19256,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-013</x:v>
       </x:c>
       <x:c r="O17" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P17" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q17" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R17" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S17" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T17" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U17" s="25" t="str">
-        <x:f>IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V17" s="25" t="str"/>
-      <x:c r="W17" s="26" t="str"/>
+        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V17" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W17" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X17" s="25" t="str">
-        <x:v>资料中出现服务响应和固定周期类表述，公开前需全部降级为合同约定。</x:v>
+        <x:v>资料中出现服务响应和固定周期类表述，公开前需全部降级为合同约定。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19262,31 +19334,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-014</x:v>
       </x:c>
       <x:c r="O18" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P18" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q18" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R18" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S18" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T18" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U18" s="25" t="str">
-        <x:f>IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V18" s="25" t="str"/>
-      <x:c r="W18" s="26" t="str"/>
+        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V18" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W18" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X18" s="25" t="str">
-        <x:v>公开时要删除“同行领先”等风险表述，只保留按工况评估。</x:v>
+        <x:v>公开时要删除“同行领先”等风险表述，只保留按工况评估。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -19333,31 +19412,38 @@
         <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-015</x:v>
       </x:c>
       <x:c r="O19" s="25" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P19" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q19" s="25" t="str">
-        <x:v>项目经验模块</x:v>
+        <x:v>网带炉现有产品页</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:f>IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V19" s="25" t="str"/>
-      <x:c r="W19" s="26" t="str"/>
+        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V19" s="25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W19" s="26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X19" s="25" t="str">
-        <x:v>更适合产品页补充，不建议单独案例页。</x:v>
+        <x:v>更适合产品页补充，不建议单独案例页。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -19416,19 +19502,21 @@
         <x:v>待确认</x:v>
       </x:c>
       <x:c r="S20" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="T20" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U20" s="25" t="str">
-        <x:f>IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
+        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="V20" s="25" t="str"/>
       <x:c r="W20" s="26" t="str"/>
       <x:c r="X20" s="25" t="str">
-        <x:v>P2，暂不进入官网案例池。</x:v>
+        <x:v>P2，暂不进入官网案例池。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -19487,19 +19575,21 @@
         <x:v>待确认</x:v>
       </x:c>
       <x:c r="S21" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="T21" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U21" s="25" t="str">
-        <x:f>IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
+        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="V21" s="25" t="str"/>
       <x:c r="W21" s="26" t="str"/>
       <x:c r="X21" s="25" t="str">
-        <x:v>P2，只能作为生产线配套资产引用。</x:v>
+        <x:v>P2，只能作为生产线配套资产引用。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -19558,19 +19648,21 @@
         <x:v>待确认</x:v>
       </x:c>
       <x:c r="S22" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="T22" s="25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U22" s="25" t="str">
-        <x:f>IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
+        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>禁发</x:v>
       </x:c>
       <x:c r="V22" s="25" t="str"/>
       <x:c r="W22" s="26" t="str"/>
       <x:c r="X22" s="25" t="str">
-        <x:v>P2，建议暂存内部资料池。</x:v>
+        <x:v>P2，建议暂存内部资料池。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -19617,31 +19709,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O23" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q23" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R23" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S23" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T23" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U23" t="str">
-        <x:f>IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V23"/>
-      <x:c r="W23"/>
+        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V23" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W23" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X23" t="str">
-        <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。</x:v>
+        <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19688,31 +19787,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O24" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q24" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R24" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S24" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T24" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U24" t="str">
-        <x:f>IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V24"/>
-      <x:c r="W24"/>
+        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V24" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W24" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X24" t="str">
-        <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。</x:v>
+        <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -19759,31 +19865,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O25" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q25" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T25" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U25" t="str">
-        <x:f>IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V25"/>
-      <x:c r="W25"/>
+        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V25" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W25" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X25" t="str">
-        <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。</x:v>
+        <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19830,31 +19943,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q26" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R26" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S26" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T26" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U26" t="str">
-        <x:f>IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V26"/>
-      <x:c r="W26"/>
+        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V26" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W26" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X26" t="str">
-        <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。</x:v>
+        <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -19901,31 +20021,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q27" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R27" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S27" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T27" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U27" t="str">
-        <x:f>IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V27"/>
-      <x:c r="W27"/>
+        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V27" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W27" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X27" t="str">
-        <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。</x:v>
+        <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -19972,31 +20099,38 @@
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
       </x:c>
       <x:c r="O28" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="Q28" t="str">
-        <x:v>内部审核；三门全过后再决定是否回填案例页</x:v>
+        <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R28" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="S28" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="T28" t="str">
-        <x:v>待确认</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U28" t="str">
-        <x:f>IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发","待审核"))</x:f>
-        <x:v>待审核</x:v>
-      </x:c>
-      <x:c r="V28"/>
-      <x:c r="W28"/>
+        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布","待审核"))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V28" t="str">
+        <x:v>钱波（行业合理性及发布确认）</x:v>
+      </x:c>
+      <x:c r="W28" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
       <x:c r="X28" t="str">
-        <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。</x:v>
+        <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。
+2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
+2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20022,7 +20156,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7329a0ad21c74a34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bd1c398d86245ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
fix(geo): align evidence maturity and index gates
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R3dc318002fad4d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="Rb08fe750f80a44a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R84d61bfce22c43de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="Ra43fb042623b4e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Ra0ccdd42f6c5487d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R30898bd54dd24629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8ad93b742dbd49fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R52e6bdfa48d642a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R269468807dba4a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Re0326d985ba64ef9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -793,20 +793,20 @@
       <x:c r="G10" s="21"/>
       <x:c r="H10" s="21"/>
     </x:row>
-    <x:row r="11" ht="30" customHeight="1">
+    <x:row r="11" ht="46.5" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>待审核事实资产</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"公司批准范围内公开（证据待补）")+COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"待审核")&amp;" 项待审核；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项可发布；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
-        <x:v>0 项待审核；21 项可发布；3 项禁发</x:v>
+        <x:f>B11&amp;" 项证据待补；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项精确值全门通过；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
+        <x:v>21 项证据待补；0 项精确值全门通过；3 项禁发</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>21 项已进入精确值可发布状态并映射到现有页面；3 项 P2 弱相关资料继续内部留存。</x:v>
+        <x:v>21 项由公司批准现有范围公开，但唐登荣技术复核及客户书面证据待补；补齐前不得新增精确值、跨页复用或站外分发。3 项 P2 弱相关资料继续内部留存。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16142,7 +16142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda89c812d5648c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03cff0d7abc4496"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18126,7 +18126,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5173fff0be4bab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2471ef082dc74d7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18192,7 +18192,7 @@
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="4" t="str">
         <x:v>24 项事实单元与三门审核
-21 项已由钱波完成行业合理性及发布确认，按现有案例、方案和产品页公开；3 项 P2 弱相关内部资料继续禁发。</x:v>
+21 项已完成公司发布批准，但唐登荣技术复核与客户书面证据仍待补；3 项 P2 弱相关资料继续禁发。现有页面可以保留，证据补齐前不得新增精确值、跨页复用或站外分发。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -18201,6 +18201,22 @@
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
+      <x:c r="Q2"/>
+      <x:c r="R2"/>
+      <x:c r="S2"/>
+      <x:c r="T2"/>
+      <x:c r="U2"/>
+      <x:c r="V2"/>
+      <x:c r="W2"/>
+      <x:c r="X2"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="24" t="str">
@@ -18323,35 +18339,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P5" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q5" s="25" t="str">
         <x:v>济宁支重轮现有案例页</x:v>
       </x:c>
       <x:c r="R5" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S5" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T5" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U5" s="25" t="str">
-        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(AND(S5="通过",OR(R5="通过",R5="待唐工复核"),T5="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V5" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W5" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W5" s="26"/>
       <x:c r="X5" s="25" t="str">
         <x:v>P0 优先，适合补强连续热处理生产线主枢纽页和工程机械行业背书；公开前需客户授权或保持脱敏。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18401,35 +18415,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P6" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q6" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R6" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S6" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T6" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U6" s="25" t="str">
-        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(AND(S6="通过",OR(R6="通过",R6="待唐工复核"),T6="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V6" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W6" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W6" s="26"/>
       <x:c r="X6" s="25" t="str">
         <x:v>P0 优先，可作为托辊网带生产线、连续热处理生产线、网带炉页面的核心项目经验。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18479,35 +18491,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P7" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q7" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R7" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S7" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T7" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U7" s="25" t="str">
-        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(AND(S7="通过",OR(R7="通过",R7="待唐工复核"),T7="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V7" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W7" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W7" s="26"/>
       <x:c r="X7" s="25" t="str">
         <x:v>多个年份和规格资料可合并为一个脱敏项目经验，避免重复案例。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -18557,35 +18567,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P8" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q8" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R8" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S8" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T8" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U8" s="25" t="str">
-        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(AND(S8="通过",OR(R8="通过",R8="待唐工复核"),T8="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V8" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W8" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W8" s="26"/>
       <x:c r="X8" s="25" t="str">
         <x:v>与网带式渗碳气氛生产线有主题接近，官网发布时应区分为“可控气氛淬火回火线”而非渗碳专页。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18635,35 +18643,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P9" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q9" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R9" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S9" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T9" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U9" s="25" t="str">
-        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(AND(S9="通过",OR(R9="通过",R9="待唐工复核"),T9="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V9" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W9" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W9" s="26"/>
       <x:c r="X9" s="25" t="str">
         <x:v>渗碳/气氛内容需克制表述，避免被理解为固定成熟标准线。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18713,35 +18719,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P10" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q10" s="25" t="str">
         <x:v>河南退火固溶现有案例页</x:v>
       </x:c>
       <x:c r="R10" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S10" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T10" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U10" s="25" t="str">
-        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(AND(S10="通过",OR(R10="通过",R10="待唐工复核"),T10="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V10" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W10" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W10" s="26"/>
       <x:c r="X10" s="25" t="str">
         <x:v>P0 优先，可支撑退火固溶生产线页面和连续热处理生产线主枢纽。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -18791,35 +18795,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P11" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q11" s="25" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R11" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S11" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T11" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U11" s="25" t="str">
-        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(AND(S11="通过",OR(R11="通过",R11="待唐工复核"),T11="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V11" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W11" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W11" s="26"/>
       <x:c r="X11" s="25" t="str">
         <x:v>源资料含客户全称，应继续脱敏；可与已公开的退洗线节能改造案例形成项目经验体系。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -18869,35 +18871,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P12" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q12" s="25" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R12" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S12" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T12" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U12" s="25" t="str">
-        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(AND(S12="通过",OR(R12="通过",R12="待唐工复核"),T12="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V12" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W12" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W12" s="26"/>
       <x:c r="X12" s="25" t="str">
         <x:v>若引用年节能或吨钢降本数据，必须使用边界说明：该数据仅适用于对应燃料结构、负荷、运行制度和改造范围。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -18947,35 +18947,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P13" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q13" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R13" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S13" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T13" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U13" s="25" t="str">
-        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(AND(S13="通过",OR(R13="通过",R13="待唐工复核"),T13="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V13" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W13" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W13" s="26"/>
       <x:c r="X13" s="25" t="str">
         <x:v>源资料含多个客户版本，可合并为一个脱敏案例或拆为项目经验模块。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -19025,35 +19023,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P14" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q14" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R14" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S14" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T14" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U14" s="25" t="str">
-        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(AND(S14="通过",OR(R14="通过",R14="待唐工复核"),T14="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V14" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W14" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W14" s="26"/>
       <x:c r="X14" s="25" t="str">
         <x:v>公开时不要承诺固定达标或固定 NOx 数值，表述为按所在地排放要求和验收口径设计。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19103,35 +19099,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P15" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q15" s="25" t="str">
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R15" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S15" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T15" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U15" s="25" t="str">
-        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(AND(S15="通过",OR(R15="通过",R15="待唐工复核"),T15="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V15" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W15" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W15" s="26"/>
       <x:c r="X15" s="25" t="str">
         <x:v>与退火固溶生产线主题高度相关，建议先用于系统页项目经验，不急于单独案例页。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19181,35 +19175,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P16" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q16" s="25" t="str">
         <x:v>箱式炉现有产品页</x:v>
       </x:c>
       <x:c r="R16" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S16" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T16" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U16" s="25" t="str">
-        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(AND(S16="通过",OR(R16="通过",R16="待唐工复核"),T16="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V16" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W16" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W16" s="26"/>
       <x:c r="X16" s="25" t="str">
         <x:v>不是铜丝自动化连续退火生产线，不能包装成铜丝连续线案例。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19259,35 +19251,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P17" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q17" s="25" t="str">
         <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R17" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S17" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T17" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U17" s="25" t="str">
-        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(AND(S17="通过",OR(R17="通过",R17="待唐工复核"),T17="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V17" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W17" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W17" s="26"/>
       <x:c r="X17" s="25" t="str">
         <x:v>资料中出现服务响应和固定周期类表述，公开前需全部降级为合同约定。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19337,35 +19327,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P18" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q18" s="25" t="str">
         <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R18" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S18" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T18" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U18" s="25" t="str">
-        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(AND(S18="通过",OR(R18="通过",R18="待唐工复核"),T18="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V18" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W18" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W18" s="26"/>
       <x:c r="X18" s="25" t="str">
         <x:v>公开时要删除“同行领先”等风险表述，只保留按工况评估。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -19415,35 +19403,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P19" s="25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q19" s="25" t="str">
         <x:v>网带炉现有产品页</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(AND(S19="通过",OR(R19="通过",R19="待唐工复核"),T19="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V19" s="25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W19" s="26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W19" s="26"/>
       <x:c r="X19" s="25" t="str">
         <x:v>更适合产品页补充，不建议单独案例页。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -19505,17 +19491,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T20" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U20" s="25" t="str">
-        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布","待审核"))</x:f>
+        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(AND(S20="通过",OR(R20="通过",R20="待唐工复核"),T20="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
-      <x:c r="V20" s="25" t="str"/>
-      <x:c r="W20" s="26" t="str"/>
+      <x:c r="V20" s="25"/>
+      <x:c r="W20" s="26"/>
       <x:c r="X20" s="25" t="str">
         <x:v>P2，暂不进入官网案例池。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19578,17 +19564,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T21" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U21" s="25" t="str">
-        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布","待审核"))</x:f>
+        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(AND(S21="通过",OR(R21="通过",R21="待唐工复核"),T21="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
-      <x:c r="V21" s="25" t="str"/>
-      <x:c r="W21" s="26" t="str"/>
+      <x:c r="V21" s="25"/>
+      <x:c r="W21" s="26"/>
       <x:c r="X21" s="25" t="str">
         <x:v>P2，只能作为生产线配套资产引用。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19651,17 +19637,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T22" s="25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U22" s="25" t="str">
-        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布","待审核"))</x:f>
+        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(AND(S22="通过",OR(R22="通过",R22="待唐工复核"),T22="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
-      <x:c r="V22" s="25" t="str"/>
-      <x:c r="W22" s="26" t="str"/>
+      <x:c r="V22" s="25"/>
+      <x:c r="W22" s="26"/>
       <x:c r="X22" s="25" t="str">
         <x:v>P2，建议暂存内部资料池。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19712,35 +19698,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P23" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q23" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R23" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S23" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T23" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U23" t="str">
-        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",OR(R23="通过",R23="待唐工复核"),T23="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V23" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W23" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W23"/>
       <x:c r="X23" t="str">
         <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19790,35 +19774,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P24" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q24" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R24" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S24" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T24" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U24" t="str">
-        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(AND(S24="通过",OR(R24="通过",R24="待唐工复核"),T24="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V24" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W24" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W24"/>
       <x:c r="X24" t="str">
         <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -19868,35 +19850,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P25" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q25" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R25" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S25" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T25" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U25" t="str">
-        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(AND(S25="通过",OR(R25="通过",R25="待唐工复核"),T25="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V25" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W25" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W25"/>
       <x:c r="X25" t="str">
         <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19946,35 +19926,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q26" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R26" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S26" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T26" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U26" t="str">
-        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(AND(S26="通过",OR(R26="通过",R26="待唐工复核"),T26="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V26" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W26" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W26"/>
       <x:c r="X26" t="str">
         <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -20024,35 +20002,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P27" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q27" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R27" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S27" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T27" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U27" t="str">
-        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",OR(R27="通过",R27="待唐工复核"),T27="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V27" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W27" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W27"/>
       <x:c r="X27" t="str">
         <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20102,35 +20078,33 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="P28" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Q28" t="str">
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R28" t="str">
-        <x:v>通过</x:v>
+        <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="S28" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T28" t="str">
-        <x:v>通过</x:v>
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
       </x:c>
       <x:c r="U28" t="str">
-        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布","待审核"))</x:f>
-        <x:v>精确值可发布</x:v>
+        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(AND(S28="通过",OR(R28="通过",R28="待唐工复核"),T28="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:v>公司批准范围内公开（证据待补）</x:v>
       </x:c>
       <x:c r="V28" t="str">
-        <x:v>钱波（行业合理性及发布确认）</x:v>
-      </x:c>
-      <x:c r="W28" t="str">
-        <x:v>2026-07-29</x:v>
-      </x:c>
+        <x:v>待安排：唐登荣</x:v>
+      </x:c>
+      <x:c r="W28"/>
       <x:c r="X28" t="str">
         <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。
-2026-07-29 钱波确认：台账当前表述均已获授权；授权仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许按本行现有口径公开；精确值仍须技术准确门通过后发布。
-2026-07-29 发布决定：钱波确认该数字符合行业常识、内容已授权并要求全部上线；此记录是负责人发布确认，不冒充唐工签审。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20140,7 +20114,7 @@
   <x:conditionalFormatting sqref="U5:U22">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="待审核"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="R5:T22">
       <x:formula1>"待确认,通过,范围表达,禁发"</x:formula1>
     </x:dataValidation>
@@ -20153,10 +20127,13 @@
     <x:dataValidation type="list" sqref="O23:P28">
       <x:formula1>"是,否,待确认"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="R5:T28">
+      <x:formula1>"待确认,通过,范围表达,禁发,待唐工复核,公司判断已在授权范围内，客户书面确认待补"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bd1c398d86245ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a8fd3cd8d54280"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20471,6 +20448,78 @@
       <x:c r="E18" s="29"/>
       <x:c r="F18" s="29"/>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>技术状态</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>待唐工复核</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>只完成行业常识初筛，尚未取得唐登荣本人技术复核记录</x:v>
+      </x:c>
+      <x:c r="D19"/>
+      <x:c r="E19" t="str">
+        <x:v>录音转写</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>经唐登荣知情同意后录音；本人只回答和确认，整理工作后置</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>客户证据状态</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>钱波批准现有公开范围，但尚无客户邮件、合同条款或会议纪要编号</x:v>
+      </x:c>
+      <x:c r="D20"/>
+      <x:c r="E20" t="str">
+        <x:v>访谈顺序</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>先补 6 条已发布口径，再问费用、验收、风险等非品牌词缺口</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>发布状态</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>公司批准范围内公开（证据待补）</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>现有页面可保留；证据补齐前不得新增精确值、跨页复用或站外分发</x:v>
+      </x:c>
+      <x:c r="D21"/>
+      <x:c r="E21" t="str">
+        <x:v>P5</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>暂缓；正式桌面端和移动端 UI 设计通过后才能施工</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>索引批次</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>青山暂缓</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>其余更新页先提交；青山案例在 6 条口径补齐并复核后单独提交</x:v>
+      </x:c>
+      <x:c r="D22"/>
+      <x:c r="E22" t="str">
+        <x:v>索引验收</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>提交成功只代表收到；继续用 nginx 日志检查实际抓取</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F2"/>

</xml_diff>

<commit_message>
fix(geo): remove authorization disclaimer wording
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R30898bd54dd24629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8ad93b742dbd49fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R52e6bdfa48d642a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R269468807dba4a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Re0326d985ba64ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R4485d86763c04d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8fcb4a5825eb44d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="Rfd703b69f5de4281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="Rbc61fff897394b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="R04e9518d7f614b8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -798,15 +798,15 @@
         <x:v>待审核事实资产</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"公司批准范围内公开（证据待补）")+COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"公开（技术复核待完成）")+COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:f>B11&amp;" 项证据待补；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项精确值全门通过；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
-        <x:v>21 项证据待补；0 项精确值全门通过；3 项禁发</x:v>
+        <x:f>B11&amp;" 项技术复核待完成；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项精确值全门通过；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
+        <x:v>21 项技术复核待完成；0 项精确值全门通过；3 项禁发</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>21 项由公司批准现有范围公开，但唐登荣技术复核及客户书面证据待补；补齐前不得新增精确值、跨页复用或站外分发。3 项 P2 弱相关资料继续内部留存。</x:v>
+        <x:v>21 项授权状态已确认，唐登荣技术复核待完成；复核前不得新增未经复核的精确值、跨页复用或站外分发。3 项 P2 弱相关资料继续内部留存。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16142,7 +16142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03cff0d7abc4496"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3a91c71937d4563"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18126,7 +18126,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2471ef082dc74d7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112f1c60817e4979"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18192,7 +18192,7 @@
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="4" t="str">
         <x:v>24 项事实单元与三门审核
-21 项已完成公司发布批准，但唐登荣技术复核与客户书面证据仍待补；3 项 P2 弱相关资料继续禁发。现有页面可以保留，证据补齐前不得新增精确值、跨页复用或站外分发。</x:v>
+21 项授权状态已确认，唐登荣技术复核待完成；3 项 P2 弱相关资料继续禁发。现有页面可以保留，技术复核完成前不得新增未经复核的精确值、跨页复用或站外分发。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -18351,11 +18351,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T5" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U5" s="25" t="str">
-        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(AND(S5="通过",OR(R5="通过",R5="待唐工复核"),T5="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(AND(S5="通过",R5="待唐工复核",T5="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V5" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18363,9 +18363,9 @@
       <x:c r="W5" s="26"/>
       <x:c r="X5" s="25" t="str">
         <x:v>P0 优先，适合补强连续热处理生产线主枢纽页和工程机械行业背书；公开前需客户授权或保持脱敏。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18427,11 +18427,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T6" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U6" s="25" t="str">
-        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(AND(S6="通过",OR(R6="通过",R6="待唐工复核"),T6="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(AND(S6="通过",R6="待唐工复核",T6="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V6" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18439,9 +18439,9 @@
       <x:c r="W6" s="26"/>
       <x:c r="X6" s="25" t="str">
         <x:v>P0 优先，可作为托辊网带生产线、连续热处理生产线、网带炉页面的核心项目经验。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18503,11 +18503,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T7" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U7" s="25" t="str">
-        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(AND(S7="通过",OR(R7="通过",R7="待唐工复核"),T7="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(AND(S7="通过",R7="待唐工复核",T7="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V7" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18515,9 +18515,9 @@
       <x:c r="W7" s="26"/>
       <x:c r="X7" s="25" t="str">
         <x:v>多个年份和规格资料可合并为一个脱敏项目经验，避免重复案例。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -18579,11 +18579,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T8" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U8" s="25" t="str">
-        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(AND(S8="通过",OR(R8="通过",R8="待唐工复核"),T8="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(AND(S8="通过",R8="待唐工复核",T8="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V8" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18591,9 +18591,9 @@
       <x:c r="W8" s="26"/>
       <x:c r="X8" s="25" t="str">
         <x:v>与网带式渗碳气氛生产线有主题接近，官网发布时应区分为“可控气氛淬火回火线”而非渗碳专页。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18655,11 +18655,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T9" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U9" s="25" t="str">
-        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(AND(S9="通过",OR(R9="通过",R9="待唐工复核"),T9="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(AND(S9="通过",R9="待唐工复核",T9="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V9" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18667,9 +18667,9 @@
       <x:c r="W9" s="26"/>
       <x:c r="X9" s="25" t="str">
         <x:v>渗碳/气氛内容需克制表述，避免被理解为固定成熟标准线。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18731,11 +18731,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T10" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U10" s="25" t="str">
-        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(AND(S10="通过",OR(R10="通过",R10="待唐工复核"),T10="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(AND(S10="通过",R10="待唐工复核",T10="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V10" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18743,9 +18743,9 @@
       <x:c r="W10" s="26"/>
       <x:c r="X10" s="25" t="str">
         <x:v>P0 优先，可支撑退火固溶生产线页面和连续热处理生产线主枢纽。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -18807,11 +18807,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T11" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U11" s="25" t="str">
-        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(AND(S11="通过",OR(R11="通过",R11="待唐工复核"),T11="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(AND(S11="通过",R11="待唐工复核",T11="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V11" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18819,9 +18819,9 @@
       <x:c r="W11" s="26"/>
       <x:c r="X11" s="25" t="str">
         <x:v>源资料含客户全称，应继续脱敏；可与已公开的退洗线节能改造案例形成项目经验体系。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -18883,11 +18883,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T12" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U12" s="25" t="str">
-        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(AND(S12="通过",OR(R12="通过",R12="待唐工复核"),T12="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(AND(S12="通过",R12="待唐工复核",T12="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V12" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18895,9 +18895,9 @@
       <x:c r="W12" s="26"/>
       <x:c r="X12" s="25" t="str">
         <x:v>若引用年节能或吨钢降本数据，必须使用边界说明：该数据仅适用于对应燃料结构、负荷、运行制度和改造范围。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -18959,11 +18959,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T13" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U13" s="25" t="str">
-        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(AND(S13="通过",OR(R13="通过",R13="待唐工复核"),T13="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(AND(S13="通过",R13="待唐工复核",T13="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V13" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -18971,9 +18971,9 @@
       <x:c r="W13" s="26"/>
       <x:c r="X13" s="25" t="str">
         <x:v>源资料含多个客户版本，可合并为一个脱敏案例或拆为项目经验模块。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -19035,11 +19035,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T14" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U14" s="25" t="str">
-        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(AND(S14="通过",OR(R14="通过",R14="待唐工复核"),T14="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(AND(S14="通过",R14="待唐工复核",T14="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V14" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19047,9 +19047,9 @@
       <x:c r="W14" s="26"/>
       <x:c r="X14" s="25" t="str">
         <x:v>公开时不要承诺固定达标或固定 NOx 数值，表述为按所在地排放要求和验收口径设计。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19111,11 +19111,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T15" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U15" s="25" t="str">
-        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(AND(S15="通过",OR(R15="通过",R15="待唐工复核"),T15="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(AND(S15="通过",R15="待唐工复核",T15="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V15" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19123,9 +19123,9 @@
       <x:c r="W15" s="26"/>
       <x:c r="X15" s="25" t="str">
         <x:v>与退火固溶生产线主题高度相关，建议先用于系统页项目经验，不急于单独案例页。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19187,11 +19187,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T16" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U16" s="25" t="str">
-        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(AND(S16="通过",OR(R16="通过",R16="待唐工复核"),T16="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(AND(S16="通过",R16="待唐工复核",T16="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V16" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19199,9 +19199,9 @@
       <x:c r="W16" s="26"/>
       <x:c r="X16" s="25" t="str">
         <x:v>不是铜丝自动化连续退火生产线，不能包装成铜丝连续线案例。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19263,11 +19263,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T17" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U17" s="25" t="str">
-        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(AND(S17="通过",OR(R17="通过",R17="待唐工复核"),T17="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(AND(S17="通过",R17="待唐工复核",T17="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V17" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19275,9 +19275,9 @@
       <x:c r="W17" s="26"/>
       <x:c r="X17" s="25" t="str">
         <x:v>资料中出现服务响应和固定周期类表述，公开前需全部降级为合同约定。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19339,11 +19339,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T18" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U18" s="25" t="str">
-        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(AND(S18="通过",OR(R18="通过",R18="待唐工复核"),T18="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(AND(S18="通过",R18="待唐工复核",T18="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V18" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19351,9 +19351,9 @@
       <x:c r="W18" s="26"/>
       <x:c r="X18" s="25" t="str">
         <x:v>公开时要删除“同行领先”等风险表述，只保留按工况评估。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -19415,11 +19415,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(AND(S19="通过",OR(R19="通过",R19="待唐工复核"),T19="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(AND(S19="通过",R19="待唐工复核",T19="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V19" s="25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19427,9 +19427,9 @@
       <x:c r="W19" s="26"/>
       <x:c r="X19" s="25" t="str">
         <x:v>更适合产品页补充，不建议单独案例页。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -19491,17 +19491,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T20" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U20" s="25" t="str">
-        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(AND(S20="通过",OR(R20="通过",R20="待唐工复核"),T20="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(AND(S20="通过",R20="待唐工复核",T20="通过"),"公开（技术复核待完成）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V20" s="25"/>
       <x:c r="W20" s="26"/>
       <x:c r="X20" s="25" t="str">
         <x:v>P2，暂不进入官网案例池。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19564,17 +19564,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T21" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U21" s="25" t="str">
-        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(AND(S21="通过",OR(R21="通过",R21="待唐工复核"),T21="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(AND(S21="通过",R21="待唐工复核",T21="通过"),"公开（技术复核待完成）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V21" s="25"/>
       <x:c r="W21" s="26"/>
       <x:c r="X21" s="25" t="str">
         <x:v>P2，只能作为生产线配套资产引用。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19637,17 +19637,17 @@
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="T22" s="25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U22" s="25" t="str">
-        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(AND(S22="通过",OR(R22="通过",R22="待唐工复核"),T22="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
+        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(AND(S22="通过",R22="待唐工复核",T22="通过"),"公开（技术复核待完成）","待审核")))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V22" s="25"/>
       <x:c r="W22" s="26"/>
       <x:c r="X22" s="25" t="str">
         <x:v>P2，建议暂存内部资料池。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
 GEO 决策：与当前热处理炉主线相关性弱，继续内部留存，不公开。</x:v>
       </x:c>
     </x:row>
@@ -19710,11 +19710,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T23" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U23" t="str">
-        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",OR(R23="通过",R23="待唐工复核"),T23="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",R23="待唐工复核",T23="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V23" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19722,9 +19722,9 @@
       <x:c r="W23"/>
       <x:c r="X23" t="str">
         <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19786,11 +19786,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T24" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U24" t="str">
-        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(AND(S24="通过",OR(R24="通过",R24="待唐工复核"),T24="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(AND(S24="通过",R24="待唐工复核",T24="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V24" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19798,9 +19798,9 @@
       <x:c r="W24"/>
       <x:c r="X24" t="str">
         <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -19862,11 +19862,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T25" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U25" t="str">
-        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(AND(S25="通过",OR(R25="通过",R25="待唐工复核"),T25="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(AND(S25="通过",R25="待唐工复核",T25="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V25" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19874,9 +19874,9 @@
       <x:c r="W25"/>
       <x:c r="X25" t="str">
         <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19938,11 +19938,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T26" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U26" t="str">
-        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(AND(S26="通过",OR(R26="通过",R26="待唐工复核"),T26="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(AND(S26="通过",R26="待唐工复核",T26="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V26" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -19950,9 +19950,9 @@
       <x:c r="W26"/>
       <x:c r="X26" t="str">
         <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -20014,11 +20014,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T27" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U27" t="str">
-        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",OR(R27="通过",R27="待唐工复核"),T27="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",R27="待唐工复核",T27="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V27" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -20026,9 +20026,9 @@
       <x:c r="W27"/>
       <x:c r="X27" t="str">
         <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20090,11 +20090,11 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="T28" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="U28" t="str">
-        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(AND(S28="通过",OR(R28="通过",R28="待唐工复核"),T28="公司判断已在授权范围内，客户书面确认待补"),"公司批准范围内公开（证据待补）","待审核")))</x:f>
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(AND(S28="通过",R28="待唐工复核",T28="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V28" t="str">
         <x:v>待安排：唐登荣</x:v>
@@ -20102,9 +20102,9 @@
       <x:c r="W28"/>
       <x:c r="X28" t="str">
         <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。
-2026-07-29 公司发布判断：钱波确认现有表述处于公司判断的授权范围内；客户书面确认记录待补。该判断仅覆盖本行现有脱敏内容，不扩大到“禁发内容”列所列客户全称、合同、图纸或其他敏感原件。
-GEO 决策：公司允许现有页面按本行口径继续公开；在唐登荣技术复核及客户书面证据补齐前，不得新增精确值、跨页面复用或站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并批准现有范围公开；这不是唐登荣技术签审，也不是客户书面确认。公开时必须保留项目级适用边界。</x:v>
+2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
+GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20128,12 +20128,12 @@
       <x:formula1>"是,否,待确认"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="R5:T28">
-      <x:formula1>"待确认,通过,范围表达,禁发,待唐工复核,公司判断已在授权范围内，客户书面确认待补"</x:formula1>
+      <x:formula1>"待确认,通过,范围表达,禁发,待唐工复核"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a8fd3cd8d54280"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a2b234ea0214cf5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20468,20 +20468,20 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>客户证据状态</x:v>
+        <x:v>授权状态</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>公司判断已在授权范围内，客户书面确认待补</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>钱波批准现有公开范围，但尚无客户邮件、合同条款或会议纪要编号</x:v>
+        <x:v>2026-07-29 钱波明确确认：当前台账内容均已授权</x:v>
       </x:c>
       <x:c r="D20"/>
       <x:c r="E20" t="str">
         <x:v>访谈顺序</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>先补 6 条已发布口径，再问费用、验收、风险等非品牌词缺口</x:v>
+        <x:v>先复核 6 条已发布口径，再问费用、验收、风险等非品牌词缺口</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -20489,10 +20489,10 @@
         <x:v>发布状态</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>公司批准范围内公开（证据待补）</x:v>
+        <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>现有页面可保留；证据补齐前不得新增精确值、跨页复用或站外分发</x:v>
+        <x:v>现有页面可保留；唐登荣技术复核完成前，不新增未经复核的精确值、跨页复用或站外分发</x:v>
       </x:c>
       <x:c r="D21"/>
       <x:c r="E21" t="str">

</xml_diff>

<commit_message>
feat(geo): publish verified project facts
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R4485d86763c04d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8fcb4a5825eb44d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="Rfd703b69f5de4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="Rbc61fff897394b4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="R04e9518d7f614b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R5d9647bc12b74606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8dc84fa6b42441b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R95f407890feb4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R64c2787391994e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Raf7ef506169a4b08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -795,18 +795,18 @@
     </x:row>
     <x:row r="11" ht="46.5" customHeight="1">
       <x:c r="A11" s="19" t="str">
-        <x:v>待审核事实资产</x:v>
+        <x:v>事实资产发布状态</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"公开（技术复核待完成）")+COUNTIF('事实单元'!$U$5:$U$28,"待审核")</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"资料参数可发布")+COUNTIF('事实单元'!$U$5:$U$28,"范围表达可发布")+COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:f>B11&amp;" 项技术复核待完成；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")&amp;" 项精确值全门通过；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
-        <x:v>21 项技术复核待完成；0 项精确值全门通过；3 项禁发</x:v>
+        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"资料参数可发布")&amp;" 项资料参数可发布；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"公开（技术复核待完成）")&amp;" 项高责任事实待补；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
+        <x:v>15 项资料参数可发布；6 项高责任事实待补；3 项禁发</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>21 项授权状态已确认，唐登荣技术复核待完成；复核前不得新增未经复核的精确值、跨页复用或站外分发。3 项 P2 弱相关资料继续内部留存。</x:v>
+        <x:v>F07–F21 已按资料确认、行业推定和禁止实绩三层口径完成分级；青山经济测算、项目周期与排放结论仍按独立高责任事实管理，资料未齐前不升级为验收实绩。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16142,7 +16142,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3a91c71937d4563"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re872a5316df14077"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18126,7 +18126,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112f1c60817e4979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d256f9e193e4b4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18318,7 +18318,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I5" s="25" t="str">
-        <x:v>处理 PC200 至 PC400 支重轮；加热炉额定温度 950℃；有效加热区约 6400×300×300mm；设计处理能力资料中出现约 500kg/h，公开时建议表述为按工件规格单独确认。</x:v>
+        <x:v>PC200–PC400 为设计适用支重轮型号范围；淬火炉额定温度 950℃；有效加热区 6400×300×300 mm；最大设计处理能力 500 kg/h，方案折算约 30 件/h。实际能力取决于单件重量、装炉方式、加热时间和生产节拍。</x:v>
       </x:c>
       <x:c r="J5" s="25" t="str">
         <x:v>支重轮规格变化、节拍要求、淬火均匀性、工件旋转与喷水分段控制、加热炉与淬火机床节拍衔接。</x:v>
@@ -18327,13 +18327,13 @@
         <x:v>生产线方案设计、连续加热炉、自动淬火机床、回火炉、喷淋冷却和控制系统配置。</x:v>
       </x:c>
       <x:c r="L5" s="25" t="str">
-        <x:v>可公开为支重轮连续热处理生产线项目经验，突出自动加热、淬火、回火、冷却联动和多规格适配。</x:v>
+        <x:v>可作为项目方案参数发布：面向 PC200–PC400 支重轮，额定温度 950℃，有效加热区 6400×300×300 mm，最大设计处理能力 500 kg/h（约 30 件/h）；必须保留实际能力边界。</x:v>
       </x:c>
       <x:c r="M5" s="25" t="str">
-        <x:v>客户全称、完整工艺图纸、PLC 程序、报价和付款条款、具体联系人信息。</x:v>
+        <x:v>不得把 500 kg/h 或约 30 件/h 写成实际验收产能；不得将 8500/10500 mm 炉体或名义长度与 6400 mm 有效加热区混写。</x:v>
       </x:c>
       <x:c r="N5" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-001</x:v>
+        <x:v>100_样本_支重轮热处理生产线_技术方案_20260519.pdf</x:v>
       </x:c>
       <x:c r="O5" s="25" t="str">
         <x:v>是</x:v>
@@ -18345,7 +18345,7 @@
         <x:v>济宁支重轮现有案例页</x:v>
       </x:c>
       <x:c r="R5" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S5" s="25" t="str">
         <x:v>通过</x:v>
@@ -18354,18 +18354,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U5" s="25" t="str">
-        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(AND(S5="通过",R5="待唐工复核",T5="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R5="禁发",S5="禁发",T5="禁发"),"禁发",IF(AND(R5="资料确认",S5="通过",T5="通过"),"资料参数可发布",IF(AND(R5="行业推定",S5="通过",T5="通过"),"范围表达可发布",IF(AND(R5="通过",S5="通过",T5="通过"),"精确值可发布",IF(AND(S5="通过",R5="待唐工复核",T5="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V5" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W5" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W5" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X5" s="25" t="str">
-        <x:v>P0 优先，适合补强连续热处理生产线主枢纽页和工程机械行业背书；公开前需客户授权或保持脱敏。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F07：F07 资料确认。PC200–PC400 为工件型号范围；950℃为额定温度，不是实际淬火工艺温度。资料确认不等于个人 reviewedBy，当前不启用唐登荣复核身份。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -18394,7 +18393,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I6" s="25" t="str">
-        <x:v>方案资料中出现正火炉有效宽度 800-1000mm、正火温度约 950℃、回火温度约 650℃、多区 PID 控温、变频调速网带；公开时不承诺固定产量。</x:v>
+        <x:v>2017 方案：正火炉有效宽度 800 mm、回火炉 1000 mm；2026 方案：正火炉工作宽度 1000 mm、回火炉 1200 mm。正火炉额定温度 950℃，回火炉额定温度 650℃；多区 PID 与网带变频调速为方案配置。</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
         <x:v>正火与回火连续衔接、快速冷却与余热利用、托辊网带同步传动、工件冷却氧化控制。</x:v>
@@ -18403,13 +18402,13 @@
         <x:v>正火炉、冷却段、回火炉、温控与传动系统方案。</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>可公开托辊网带正火回火连续线的工艺链、设备组成、节拍调节和冷却段设计思路。</x:v>
+        <x:v>资料参数可按年份和炉段分别发布。碳钢/低合金钢适用范围及正火 880–940℃、高温回火 550–650℃只能写为行业典型工况，最终按材料牌号、截面和性能要求确定。</x:v>
       </x:c>
       <x:c r="M6" s="25" t="str">
-        <x:v>客户全称、精确报价、完整布置图、供应商清单、验收细则。</x:v>
+        <x:v>不得把不同年份、不同炉段的 800/1000/1200 mm 合并成一个项目的可选参数；不得把典型工艺或方案配置写成项目验收实绩。</x:v>
       </x:c>
       <x:c r="N6" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-002</x:v>
+        <x:v>100_样本_托辊式网带正火回火生产线_技术方案_20170902.pdf；100_样本_托辊网带正火回火生产线_技术方案_20260519.pdf</x:v>
       </x:c>
       <x:c r="O6" s="25" t="str">
         <x:v>是</x:v>
@@ -18421,7 +18420,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R6" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S6" s="25" t="str">
         <x:v>通过</x:v>
@@ -18430,18 +18429,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U6" s="25" t="str">
-        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(AND(S6="通过",R6="待唐工复核",T6="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R6="禁发",S6="禁发",T6="禁发"),"禁发",IF(AND(R6="资料确认",S6="通过",T6="通过"),"资料参数可发布",IF(AND(R6="行业推定",S6="通过",T6="通过"),"范围表达可发布",IF(AND(R6="通过",S6="通过",T6="通过"),"精确值可发布",IF(AND(S6="通过",R6="待唐工复核",T6="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V6" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W6" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W6" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X6" s="25" t="str">
-        <x:v>P0 优先，可作为托辊网带生产线、连续热处理生产线、网带炉页面的核心项目经验。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F08：F08 混合口径：宽度与额定温度属于资料确认；材料及典型温度范围属于行业推定。官网须在同一事实单元内明确分层。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -18470,7 +18468,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I7" s="25" t="str">
-        <x:v>资料中出现 RCWT 系列方案、有效宽度约 800-850mm、淬火炉额定温度 950℃、回火炉 650℃、网带速度约 30-300mm/min 或 30-250mm/min，具体需按工件单独确认。</x:v>
+        <x:v>2020 RCWT-360/220-9/6：淬火炉有效宽度 850 mm、回火炉 1000 mm、速度 30–250 mm/min；2026 RCWT-250/200-9/6：淬火炉有效宽度 800 mm、回火炉 1000 mm、速度 50–300 mm/min。额定温度分别为 950℃、650℃。</x:v>
       </x:c>
       <x:c r="J7" s="25" t="str">
         <x:v>长炉膛网带承载与托辊支撑、油槽提升与清洗段衔接、气氛/碳势控制、工件堆料状态对产能的影响。</x:v>
@@ -18479,13 +18477,13 @@
         <x:v>生产线工艺方案、淬火炉、油槽提升、清洗机、回火炉、气氛控制和电气联锁。</x:v>
       </x:c>
       <x:c r="L7" s="25" t="str">
-        <x:v>可公开为托辊网带淬火回火生产线项目经验，突出托辊支撑、连续输送和配套清洗/回火联动。</x:v>
+        <x:v>按型号和年份拆开发布，不合并成通用参数；已将原“30–300 mm/min”纠正为 2026 方案的“50–300 mm/min”。</x:v>
       </x:c>
       <x:c r="M7" s="25" t="str">
-        <x:v>客户全称、内部报价、完整控制逻辑、油槽细部图、供应商清单。</x:v>
+        <x:v>不得把两个型号的宽度和速度拼成一组固定参数；950℃、650℃不得描述为实际工艺温度。</x:v>
       </x:c>
       <x:c r="N7" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-003</x:v>
+        <x:v>100_样本_托辊式网带炉热处理生产线_技术方案_20200119.pdf；100_样本_托辊式网带炉热处理生产线（151）_技术方案_20260519.pdf</x:v>
       </x:c>
       <x:c r="O7" s="25" t="str">
         <x:v>是</x:v>
@@ -18497,7 +18495,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R7" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S7" s="25" t="str">
         <x:v>通过</x:v>
@@ -18506,18 +18504,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U7" s="25" t="str">
-        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(AND(S7="通过",R7="待唐工复核",T7="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R7="禁发",S7="禁发",T7="禁发"),"禁发",IF(AND(R7="资料确认",S7="通过",T7="通过"),"资料参数可发布",IF(AND(R7="行业推定",S7="通过",T7="通过"),"范围表达可发布",IF(AND(R7="通过",S7="通过",T7="通过"),"精确值可发布",IF(AND(S7="通过",R7="待唐工复核",T7="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V7" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W7" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W7" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X7" s="25" t="str">
-        <x:v>多个年份和规格资料可合并为一个脱敏项目经验，避免重复案例。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F09：F09 资料确认。官网和内部去重资料中的 30–300 mm/min 均应修正为 50–300 mm/min。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -18546,7 +18543,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I8" s="25" t="str">
-        <x:v>资料中出现 RCWT-75/45-9/6 型，淬火炉工作尺寸约 400×3200mm，回火炉约 400×5600mm，额定温度 950℃，生产能力约 150kg/h，网带速度约 30-250mm/min。</x:v>
+        <x:v>RCWT-75/45-9/6：淬火段名义 75 kW、回火段名义 45 kW（方案实际增容至 60 kW）；额定温度通常为 950℃/650℃；有效尺寸 400×3200 mm / 400×5600 mm；网带速度 30–250 mm/min。最大设计能力约 150 kg/h，计算条件为 0.4 m×0.25 m/min×60×25 kg/㎡。</x:v>
       </x:c>
       <x:c r="J8" s="25" t="str">
         <x:v>小件保护气氛加热、油烟隔离、落料通道密封、炉内碳势或气氛稳定、清洗回火节拍衔接。</x:v>
@@ -18555,13 +18552,13 @@
         <x:v>保护气氛网带淬火炉、淬火槽、清洗机、回火炉、气氛控制和温控系统方案。</x:v>
       </x:c>
       <x:c r="L8" s="25" t="str">
-        <x:v>可公开可控气氛托辊网带生产线的设备组成、保护气氛、淬火清洗回火联动。</x:v>
+        <x:v>尺寸、速度和带计算条件的设计能力可发布；速度工况只能写为典型选型说明，实际产能按工件、铺料和加热时间确定。</x:v>
       </x:c>
       <x:c r="M8" s="25" t="str">
-        <x:v>氧探头/碳势控制细节、完整电控图、客户全称、报价和付款条款。</x:v>
+        <x:v>不得把 150 kg/h 写成验收产能；不得把 75/45 型号功率与方案实际 60 kW 回火段配置混为同一口径。</x:v>
       </x:c>
       <x:c r="N8" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-004</x:v>
+        <x:v>100_样本_可控气氛托辊网带炉生产线_技术方案_20260512.pdf</x:v>
       </x:c>
       <x:c r="O8" s="25" t="str">
         <x:v>是</x:v>
@@ -18573,7 +18570,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R8" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S8" s="25" t="str">
         <x:v>通过</x:v>
@@ -18582,18 +18579,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U8" s="25" t="str">
-        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(AND(S8="通过",R8="待唐工复核",T8="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R8="禁发",S8="禁发",T8="禁发"),"禁发",IF(AND(R8="资料确认",S8="通过",T8="通过"),"资料参数可发布",IF(AND(R8="行业推定",S8="通过",T8="通过"),"范围表达可发布",IF(AND(R8="通过",S8="通过",T8="通过"),"精确值可发布",IF(AND(S8="通过",R8="待唐工复核",T8="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V8" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W8" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W8" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X8" s="25" t="str">
-        <x:v>与网带式渗碳气氛生产线有主题接近，官网发布时应区分为“可控气氛淬火回火线”而非渗碳专页。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F10：F10 资料确认 + 行业推定。理论能力公式必须与数字同页出现，避免脱离铺料面密度被引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -18622,7 +18618,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I9" s="25" t="str">
-        <x:v>资料中出现有效加热区约 9300×1000×100mm，最高工作温度 950℃，加热功率约 300kW，生产量资料按件/天表述；公开时需标注仅适用于该工件和节拍。</x:v>
+        <x:v>有效加热区 9300×1000×100 mm；渗碳气氛淬火加热炉段功率 300 kW；最高工作温度 950℃。典型设计能力约 5000 件/24 h，最大工况约 6000 件/24 h，后者较前者高约 20%。</x:v>
       </x:c>
       <x:c r="J9" s="25" t="str">
         <x:v>渗碳气氛密封、油烟进入加热区控制、托辊与网带寿命、淬火槽温度与提升机构联动。</x:v>
@@ -18631,13 +18627,13 @@
         <x:v>渗碳气氛加热炉、淬火槽、托辊网带输送、气氛管路和控制系统。</x:v>
       </x:c>
       <x:c r="L9" s="25" t="str">
-        <x:v>可公开为网带式渗碳气氛热处理生产线项目经验，突出气氛密封、双层托辊、淬火槽联动。</x:v>
+        <x:v>尺寸、炉段功率、最高工作温度和项目设计能力可发布；6000 件/24 h 只能写为提高速度、铺料密度或利用率后的最大设计工况。</x:v>
       </x:c>
       <x:c r="M9" s="25" t="str">
-        <x:v>具体客户、产量承诺、气氛配比细节、报价单、工艺配方和图纸。</x:v>
+        <x:v>不得把 300 kW 写成全线总功率；不得把 5000/6000 件写成实际日产量；未知单件重量时不得换算为 kg/h。</x:v>
       </x:c>
       <x:c r="N9" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-005</x:v>
+        <x:v>100_样本_网带式渗碳气氛热处理生产线_技术方案_2018.pdf</x:v>
       </x:c>
       <x:c r="O9" s="25" t="str">
         <x:v>是</x:v>
@@ -18649,7 +18645,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R9" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S9" s="25" t="str">
         <x:v>通过</x:v>
@@ -18658,18 +18654,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U9" s="25" t="str">
-        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(AND(S9="通过",R9="待唐工复核",T9="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R9="禁发",S9="禁发",T9="禁发"),"禁发",IF(AND(R9="资料确认",S9="通过",T9="通过"),"资料参数可发布",IF(AND(R9="行业推定",S9="通过",T9="通过"),"范围表达可发布",IF(AND(R9="通过",S9="通过",T9="通过"),"精确值可发布",IF(AND(S9="通过",R9="待唐工复核",T9="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V9" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W9" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W9" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X9" s="25" t="str">
-        <x:v>渗碳/气氛内容需克制表述，避免被理解为固定成熟标准线。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F11：F11 资料确认 + 设计边界。件/天必须同时说明工件规格、铺料密度、网带速度和连续运行时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -18698,7 +18693,7 @@
         <x:v>设备分包 / 生产线</x:v>
       </x:c>
       <x:c r="I10" s="25" t="str">
-        <x:v>资料中出现 850mm 热轧不锈钢连续退火钝化线、退火温度约 1050-1150℃、炉温最高可至 1300℃、退火炉主体长度约 130m、带速与 TV 值按材料规格计算。</x:v>
+        <x:v>850 mm 为名义机组规格；实际带宽 480–750 mm、厚度 1.6–4.0 mm，面向 200/300 系不锈钢。带钢退火温度 1050–1150℃；1300℃为高温炉段最高设计能力。炉体约 130 m（40 m 预热 + 36 m 快速加热 + 54 m 均热），不含约 45 m 冷却/固溶段。设计 TV≈190 m·mm/min。</x:v>
       </x:c>
       <x:c r="J10" s="25" t="str">
         <x:v>带材高速连续退火固溶、敏化区快速通过、分段冷却、张力与板形控制、燃烧与余热利用。</x:v>
@@ -18707,13 +18702,13 @@
         <x:v>退火固溶段工艺设计、炉体与冷却段设备、燃烧与控制系统、安装调试配合。</x:v>
       </x:c>
       <x:c r="L10" s="25" t="str">
-        <x:v>可公开为不锈钢连续退洗线退火固溶段设备项目经验，强调工程总包配套和退火固溶段系统设计。</x:v>
+        <x:v>可作为河南 850 mm 退火固溶线项目方案参数发布；代表工况 1.8 mm×100 m/min=TV180，只用于解释 TV 计算。</x:v>
       </x:c>
       <x:c r="M10" s="25" t="str">
-        <x:v>买方/总包全称、钢种明细、完整技术协议、布置图、材料清单、报价与合同边界。</x:v>
+        <x:v>不得把 850 mm 写成实际带宽；不得把 1300℃写成带钢目标温度；不得把 130 m 写成含冷却段的整线长度。</x:v>
       </x:c>
       <x:c r="N10" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-006</x:v>
+        <x:v>100_样本_连续退洗线退火固溶段设备_技术方案_20170726.doc</x:v>
       </x:c>
       <x:c r="O10" s="25" t="str">
         <x:v>是</x:v>
@@ -18725,7 +18720,7 @@
         <x:v>河南退火固溶现有案例页</x:v>
       </x:c>
       <x:c r="R10" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S10" s="25" t="str">
         <x:v>通过</x:v>
@@ -18734,18 +18729,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U10" s="25" t="str">
-        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(AND(S10="通过",R10="待唐工复核",T10="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R10="禁发",S10="禁发",T10="禁发"),"禁发",IF(AND(R10="资料确认",S10="通过",T10="通过"),"资料参数可发布",IF(AND(R10="行业推定",S10="通过",T10="通过"),"范围表达可发布",IF(AND(R10="通过",S10="通过",T10="通过"),"精确值可发布",IF(AND(S10="通过",R10="待唐工复核",T10="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V10" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W10" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W10" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X10" s="25" t="str">
-        <x:v>P0 优先，可支撑退火固溶生产线页面和连续热处理生产线主枢纽。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F12：F12 资料确认。已有河南案例页承载，修正名义规格、实际带宽、炉段长度与 TV 口径。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -18774,7 +18768,7 @@
         <x:v>生产线 / 设备分包</x:v>
       </x:c>
       <x:c r="I11" s="25" t="str">
-        <x:v>资料中出现 1250mm 连续退洗线、单线退火固溶段、工艺速度约 40-45m/min、钢卷重量 Max28t、退火工艺段约 105m；公开时只保留范围和系统能力描述。</x:v>
+        <x:v>1250 mm 为名义机组规格及最大带宽；实际带宽 800–1250 mm、厚度 2.5–4.0 mm，适用 AISI 200/300 系不锈钢。额定工艺速度 40 m/min、最大 45 m/min；代表工况 1250×3.0 mm、TV120；带钢温度约 1080–1180℃；最大设计钢卷重量 28 t；加热/均热段约 105 m，不含固溶冷却段。</x:v>
       </x:c>
       <x:c r="J11" s="25" t="str">
         <x:v>宽带不锈钢连续处理、退火固溶段设备供货边界、圆盘辊/托辊快速更换、板温监控和多系统联动。</x:v>
@@ -18783,13 +18777,13 @@
         <x:v>退火固溶段设备、燃烧系统、冷却烘干系统、托辊与电控系统配套。</x:v>
       </x:c>
       <x:c r="L11" s="25" t="str">
-        <x:v>可脱敏为 1250mm 不锈钢连续退洗线退火固溶段项目经验。</x:v>
+        <x:v>可作为 1250 mm 连续退洗线项目方案参数发布，逐项标明名义规格、实际范围、额定/最大速度和炉段边界。</x:v>
       </x:c>
       <x:c r="M11" s="25" t="str">
-        <x:v>客户全称、材料清单重量、控制柜规格、供应商品牌、合同条款、报价和付款信息。</x:v>
+        <x:v>不得把 1250 mm 当成所有带钢的实际宽度；不得把 105 m 写成含固溶冷却段的整线长度；不得写成实际验收产量。</x:v>
       </x:c>
       <x:c r="N11" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-007</x:v>
+        <x:v>100_样本_鼎信科技连续退洗线（二期）退火固溶段设备_技术方案_20140923.doc</x:v>
       </x:c>
       <x:c r="O11" s="25" t="str">
         <x:v>是</x:v>
@@ -18801,7 +18795,7 @@
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R11" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S11" s="25" t="str">
         <x:v>通过</x:v>
@@ -18810,18 +18804,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U11" s="25" t="str">
-        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(AND(S11="通过",R11="待唐工复核",T11="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R11="禁发",S11="禁发",T11="禁发"),"禁发",IF(AND(R11="资料确认",S11="通过",T11="通过"),"资料参数可发布",IF(AND(R11="行业推定",S11="通过",T11="通过"),"范围表达可发布",IF(AND(R11="通过",S11="通过",T11="通过"),"精确值可发布",IF(AND(S11="通过",R11="待唐工复核",T11="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V11" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W11" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W11" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X11" s="25" t="str">
-        <x:v>源资料含客户全称，应继续脱敏；可与已公开的退洗线节能改造案例形成项目经验体系。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F13：F13 资料确认。可支撑连续退洗线案例的设备能力描述，但不替代 F02–F04 的经济测算底稿。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -18850,7 +18843,7 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I12" s="25" t="str">
-        <x:v>资料中出现 1250mm 连续退洗线三线改造、冷煤气替代天然气、双交叉限幅控制、节能测算数据。公开引用具体数据时必须标注只适用于该项目工况。</x:v>
+        <x:v>三条 1250 mm 连续退洗线由天然气改为冷煤气；热值与耗量换算口径为天然气 8500 kcal/Nm³、约 30 Nm³/t，对比冷煤气 1450 kcal/Nm³、约 180–200 Nm³/t。冷煤气总设计量 17150 Nm³/h，接口压力 20±3 kPa；采用双交叉限幅控制。</x:v>
       </x:c>
       <x:c r="J12" s="25" t="str">
         <x:v>低热值冷煤气替代、燃气管径与流量放大、排烟能力提升、炉膛维护与燃烧控制同步改造。</x:v>
@@ -18859,13 +18852,13 @@
         <x:v>燃烧系统升级、管路阀组、低 NOx 烧嘴、控制系统优化、炉膛检修和固溶段配套改造。</x:v>
       </x:c>
       <x:c r="L12" s="25" t="str">
-        <x:v>可公开为老旧连续退洗线节能改造项目经验，重点讲燃烧系统和控制系统升级。</x:v>
+        <x:v>可发布项目燃料转换、流量压力、控制方法和改造范围；热平衡复算、管阀压力复核、烧嘴选型、氧量修正、排烟炉压匹配、安全联锁和利旧评估可写成通用方法。</x:v>
       </x:c>
       <x:c r="M12" s="25" t="str">
-        <x:v>客户全称、完整能耗台账、内部节能计算表、燃气参数全表、报价和合同条款。</x:v>
+        <x:v>不得把冷煤气、DN700、104 套烧嘴、10 区、75 kW 风机、三条线和 2015 年经济参数外推成通用配置；不得据此自动认定 F02–F04 经济结果为实绩。</x:v>
       </x:c>
       <x:c r="N12" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-008</x:v>
+        <x:v>100_样本_一期连续退洗线退火炉燃烧系统及固溶段设备技术改造_技术方案_20151009.doc</x:v>
       </x:c>
       <x:c r="O12" s="25" t="str">
         <x:v>是</x:v>
@@ -18877,7 +18870,7 @@
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R12" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S12" s="25" t="str">
         <x:v>通过</x:v>
@@ -18886,18 +18879,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U12" s="25" t="str">
-        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(AND(S12="通过",R12="待唐工复核",T12="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R12="禁发",S12="禁发",T12="禁发"),"禁发",IF(AND(R12="资料确认",S12="通过",T12="通过"),"资料参数可发布",IF(AND(R12="行业推定",S12="通过",T12="通过"),"范围表达可发布",IF(AND(R12="通过",S12="通过",T12="通过"),"精确值可发布",IF(AND(S12="通过",R12="待唐工复核",T12="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V12" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W12" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W12" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X12" s="25" t="str">
-        <x:v>若引用年节能或吨钢降本数据，必须使用边界说明：该数据仅适用于对应燃料结构、负荷、运行制度和改造范围。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F14：F14 资料确认。技术方案可确认三条 1250 mm 及燃料改造口径，但 7,644 万元/年、63.7 元/吨、120 万吨/年仍按项目测算事实单独管理。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -18926,7 +18918,7 @@
         <x:v>生产线 / 设备分包</x:v>
       </x:c>
       <x:c r="I13" s="25" t="str">
-        <x:v>资料中出现 850/1250 设备规格书、退火炉由预热段和 4 个加热段组成，燃烧区约 8 区控制，带钢退火温度通常 700-1200℃，冷却至约 80℃以下。</x:v>
+        <x:v>850 与 1250 为两个 HAPL 项目：2021 青拓 850 项目、2024 无锡硕阳 1250 项目。炉体为预热段 + 4 个加热段，每个加热段分 2 个控温区，约 8 区控制；700–1200℃为工艺覆盖范围。冷却/干燥段出口以红外测温，目标低于 80℃；验收条件为同规格连续稳定生产 3 卷时考核。</x:v>
       </x:c>
       <x:c r="J13" s="25" t="str">
         <x:v>连续带钢退火炉系统边界大、板形与冷却速率控制、预热空气燃烧、圆盘辊或提升辊支撑、自动化和安全联锁。</x:v>
@@ -18935,13 +18927,13 @@
         <x:v>退火炉设备方案、燃烧系统、冷却干燥段、现场仪表和控制系统配套。</x:v>
       </x:c>
       <x:c r="L13" s="25" t="str">
-        <x:v>可公开为热轧退火酸洗项目退火炉项目经验，突出预热、加热、冷却、干燥系统级能力。</x:v>
+        <x:v>可按两个项目分别发布炉体结构、温区和项目考核条件，不合并成一个项目。</x:v>
       </x:c>
       <x:c r="M13" s="25" t="str">
-        <x:v>客户全称、设备布置图、主要供应商、验收细则、详细电机表和报价。</x:v>
+        <x:v>不得把 700–1200℃写成设备最高能力；不得把两个项目混为一条通用规格；无验收记录时不得写成已经达到低于 80℃。</x:v>
       </x:c>
       <x:c r="N13" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-009</x:v>
+        <x:v>100_样本_青拓不锈钢热轧退火酸洗项目退火炉_技术方案_2021.doc；100_样本_无锡硕阳热轧退火酸洗项目退火炉_技术方案_20240423.doc</x:v>
       </x:c>
       <x:c r="O13" s="25" t="str">
         <x:v>是</x:v>
@@ -18953,7 +18945,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R13" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S13" s="25" t="str">
         <x:v>通过</x:v>
@@ -18962,18 +18954,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U13" s="25" t="str">
-        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(AND(S13="通过",R13="待唐工复核",T13="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R13="禁发",S13="禁发",T13="禁发"),"禁发",IF(AND(R13="资料确认",S13="通过",T13="通过"),"资料参数可发布",IF(AND(R13="行业推定",S13="通过",T13="通过"),"范围表达可发布",IF(AND(R13="通过",S13="通过",T13="通过"),"精确值可发布",IF(AND(S13="通过",R13="待唐工复核",T13="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V13" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W13" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W13" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X13" s="25" t="str">
-        <x:v>源资料含多个客户版本，可合并为一个脱敏案例或拆为项目经验模块。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F15：F15 资料确认。官网应明确两个不同年份、不同机组规格项目。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -19002,7 +18993,7 @@
         <x:v>生产线 / 新建</x:v>
       </x:c>
       <x:c r="I14" s="25" t="str">
-        <x:v>资料中出现有效尺寸约 2.5×1.6×0.8m，设备数量 2 台，最高温度 950℃，每台 4 套 250kW 低氮烧嘴，换热后助燃空气约 200-300℃。</x:v>
+        <x:v>同一生产线含 2 台燃气加热炉；单台有效工作尺寸 2500×1600×800 mm，每台 4 套 250 kW 级低氮天然气烧嘴，燃烧装机能力约 1000 kW。助燃空气设计预热至 200–300℃。</x:v>
       </x:c>
       <x:c r="J14" s="25" t="str">
         <x:v>低 NOx 燃烧、炉压微压控制、燃气安全联锁、余热回收、温度均匀性和环保要求之间的平衡。</x:v>
@@ -19011,13 +19002,13 @@
         <x:v>燃气加热炉、封闭冷却箱、低氮燃烧系统、炉压控制、排烟余热回收和温控记录系统。</x:v>
       </x:c>
       <x:c r="L14" s="25" t="str">
-        <x:v>可公开低氮燃气加热炉生产线项目经验，强调低氮燃烧方案和燃气安全控制。</x:v>
+        <x:v>尺寸、数量、烧嘴级别和燃烧输入能力可作为方案参数发布；NOx 只能写“按所在地排放要求设计，并以有资质现场检测为准”。</x:v>
       </x:c>
       <x:c r="M14" s="25" t="str">
-        <x:v>客户全称、项目详细排放验收报告、燃气管路图、报价和付款条款。</x:v>
+        <x:v>不得把 1000 kW 写成电气功率；不得把 200–300℃写成实测温度；不得写“实测 NOx 低于 150–200 mg/Nm³”或固定达标。</x:v>
       </x:c>
       <x:c r="N14" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-010</x:v>
+        <x:v>100_样本_低氮氧化物燃气加热炉生产线_技术方案_20200811.pdf</x:v>
       </x:c>
       <x:c r="O14" s="25" t="str">
         <x:v>是</x:v>
@@ -19029,7 +19020,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R14" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S14" s="25" t="str">
         <x:v>通过</x:v>
@@ -19038,18 +19029,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U14" s="25" t="str">
-        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(AND(S14="通过",R14="待唐工复核",T14="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R14="禁发",S14="禁发",T14="禁发"),"禁发",IF(AND(R14="资料确认",S14="通过",T14="通过"),"资料参数可发布",IF(AND(R14="行业推定",S14="通过",T14="通过"),"范围表达可发布",IF(AND(R14="通过",S14="通过",T14="通过"),"精确值可发布",IF(AND(S14="通过",R14="待唐工复核",T14="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V14" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W14" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W14" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X14" s="25" t="str">
-        <x:v>公开时不要承诺固定达标或固定 NOx 数值，表述为按所在地排放要求和验收口径设计。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F16：F16 核心参数资料确认，NOx 150–200 mg/Nm³仅为行业设计目标，不在官网作为项目实绩发布。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -19078,7 +19068,7 @@
         <x:v>生产线</x:v>
       </x:c>
       <x:c r="I15" s="25" t="str">
-        <x:v>资料中出现 750t/d 双带炉、带钢宽度约 485-610mm，厚度约 2.0-5.5mm，工艺速度约 26.6m/min，炉子段约 110m，烧嘴总功率资料中有配置值。</x:v>
+        <x:v>单台炉合同设计/保证能力 750 t/d；代表计算条件为 J3A、2.3×600 mm、双带、26.6 m/min。带钢宽 485–610 mm；原料厚 2.0–3.5 mm、产品厚 2.0–5.5 mm。炉体约 110 m（25.6 m 预热 + 84.4 m 加热/均热），含水冷挤干干燥约 125.4 m。资料反推 106 套烧嘴，装机约 16680 kW，设计需用约 10500 kW。</x:v>
       </x:c>
       <x:c r="J15" s="25" t="str">
         <x:v>双带无张力退火、预热和均热段组织、带钢冷却至规定出口温度、收放卷和纠偏边界协同。</x:v>
@@ -19087,13 +19077,13 @@
         <x:v>连续退火炉、燃烧系统、冷却烘干段、温控和联锁系统，配合产线边界实施。</x:v>
       </x:c>
       <x:c r="L15" s="25" t="str">
-        <x:v>可公开为不锈钢连续退火炉双带炉项目经验，突出带材连续退火系统能力。</x:v>
+        <x:v>可发布合同设计能力、代表计算条件、材料范围和长度边界；烧嘴数量应说明为按参数与总数核对后的方案口径。</x:v>
       </x:c>
       <x:c r="M15" s="25" t="str">
-        <x:v>客户全称、厂区地址、详细年产量和产量计算表、供应商品牌、报价和合同条款。</x:v>
+        <x:v>不得把 750 t/d 写成实际日产量；不得把原料厚度与产品厚度混写；第六区 17 套疑似文字错误，不直接作为精确事实引用。</x:v>
       </x:c>
       <x:c r="N15" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P0-011</x:v>
+        <x:v>100_样本_不锈钢连续退火炉（双带炉）_技术方案_20220808.doc</x:v>
       </x:c>
       <x:c r="O15" s="25" t="str">
         <x:v>是</x:v>
@@ -19105,7 +19095,7 @@
         <x:v>连续热处理生产线现有方案页</x:v>
       </x:c>
       <x:c r="R15" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S15" s="25" t="str">
         <x:v>通过</x:v>
@@ -19114,18 +19104,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U15" s="25" t="str">
-        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(AND(S15="通过",R15="待唐工复核",T15="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R15="禁发",S15="禁发",T15="禁发"),"禁发",IF(AND(R15="资料确认",S15="通过",T15="通过"),"资料参数可发布",IF(AND(R15="行业推定",S15="通过",T15="通过"),"范围表达可发布",IF(AND(R15="通过",S15="通过",T15="通过"),"精确值可发布",IF(AND(S15="通过",R15="待唐工复核",T15="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V15" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W15" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W15" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X15" s="25" t="str">
-        <x:v>与退火固溶生产线主题高度相关，建议先用于系统页项目经验，不急于单独案例页。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F17：F17 资料确认。第六区采用 18 套仅作为资料校核结论，官网优先发布总数与总装机口径，不展开疑似错字。</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -19154,7 +19143,7 @@
         <x:v>新建 / 单炉设备组</x:v>
       </x:c>
       <x:c r="I16" s="25" t="str">
-        <x:v>资料中出现 4 台炉体，额定温度 700℃，使用温度约 550-700℃，每室约 200kW，装料有效尺寸约 Φ1710×1600mm，PLC 控制。</x:v>
+        <x:v>一套铜合金线材退火系统包含 4 个炉室；额定温度 700℃、使用 550–700℃；每室 200 kW、4 室合计 800 kW，整套系统含辅助设备不超过约 860 kW。装料有效区 Φ1710×1600 mm；炉室有效尺寸 2100×2000×1800 mm；氮气保护；每室 7.5 kW 顶部循环风机；S7-1200 PLC、14 英寸 HMI、每室 2 区 PID。</x:v>
       </x:c>
       <x:c r="J16" s="25" t="str">
         <x:v>铜合金线材装料方式、保护气氛、热风循环均匀性、自动装卸料小车与多炉联动。</x:v>
@@ -19163,13 +19152,13 @@
         <x:v>室式退火炉、热风循环、氮气管路、自动装卸料和控制系统方案。</x:v>
       </x:c>
       <x:c r="L16" s="25" t="str">
-        <x:v>可脱敏用于铜材/线材退火相关项目经验，说明苏能具备铜合金线材退火设备能力。</x:v>
+        <x:v>可在箱式炉现有产品页写为“项目方案配置”，明确是一套系统、四个炉室。</x:v>
       </x:c>
       <x:c r="M16" s="25" t="str">
-        <x:v>客户全称、车间位置、详细控制参数、报价单、联系人和付款条款。</x:v>
+        <x:v>不得把四个炉室写成四个无关项目；不得把方案配置写成已经验收的实绩。</x:v>
       </x:c>
       <x:c r="N16" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-012</x:v>
+        <x:v>100_样本_芜湖楚江合金铜材有限公司 室式电加热退火炉_技术方案_20260511.pdf</x:v>
       </x:c>
       <x:c r="O16" s="25" t="str">
         <x:v>是</x:v>
@@ -19181,7 +19170,7 @@
         <x:v>箱式炉现有产品页</x:v>
       </x:c>
       <x:c r="R16" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S16" s="25" t="str">
         <x:v>通过</x:v>
@@ -19190,18 +19179,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U16" s="25" t="str">
-        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(AND(S16="通过",R16="待唐工复核",T16="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R16="禁发",S16="禁发",T16="禁发"),"禁发",IF(AND(R16="资料确认",S16="通过",T16="通过"),"资料参数可发布",IF(AND(R16="行业推定",S16="通过",T16="通过"),"范围表达可发布",IF(AND(R16="通过",S16="通过",T16="通过"),"精确值可发布",IF(AND(S16="通过",R16="待唐工复核",T16="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V16" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W16" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W16" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X16" s="25" t="str">
-        <x:v>不是铜丝自动化连续退火生产线，不能包装成铜丝连续线案例。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F18：F18 资料确认。官网不得使用“已验收项目”措辞。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -19230,7 +19218,7 @@
         <x:v>新建 / 改造，待按源文件确认</x:v>
       </x:c>
       <x:c r="I17" s="25" t="str">
-        <x:v>资料中出现 10m×3m×2.2m 台车式轴承钢丝球化退火炉相关方案；具体温度、装炉量和改造边界需二次核对。</x:v>
+        <x:v>2017 新建台车式轴承钢丝球化退火炉：有效炉膛 10×3×2.2 m；最高设计温度 850℃；常用球化退火 790–810℃；最大装炉量 30 t（不含工装和垫铁）；有效区炉温均匀性设计要求 ≤±5℃。2018 资料为同尺寸炉型燃烧控制改造方案。</x:v>
       </x:c>
       <x:c r="J17" s="25" t="str">
         <x:v>钢丝盘卷或线材装炉、球化退火工艺曲线、温度均匀性和炉内承载方式。</x:v>
@@ -19239,13 +19227,13 @@
         <x:v>台车式球化退火炉方案、制造或改造、安装调试配合。</x:v>
       </x:c>
       <x:c r="L17" s="25" t="str">
-        <x:v>可用于台车炉页面项目经验模块，说明台车炉可覆盖轴承钢丝球化退火场景。</x:v>
+        <x:v>产品页只采用 2017 新炉参数；典型 GCr15 工艺曲线、组织 2–4 级和 179–207 HBW 只能作为行业典型说明。</x:v>
       </x:c>
       <x:c r="M17" s="25" t="str">
-        <x:v>客户全称、精确工艺曲线、服务响应承诺、报价和合同周期。</x:v>
+        <x:v>不得把 2017 新炉与 2018 改造混成一个项目；不得把典型曲线、组织、硬度或均匀性要求写成该项目实际验收结果。</x:v>
       </x:c>
       <x:c r="N17" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-013</x:v>
+        <x:v>100_样本_台车式轴承钢丝球化退火炉_技术方案_20170421.pdf；100_样本_台车式轴承钢丝球化退火炉_技术方案_20180226.pdf</x:v>
       </x:c>
       <x:c r="O17" s="25" t="str">
         <x:v>是</x:v>
@@ -19257,7 +19245,7 @@
         <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R17" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S17" s="25" t="str">
         <x:v>通过</x:v>
@@ -19266,18 +19254,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U17" s="25" t="str">
-        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(AND(S17="通过",R17="待唐工复核",T17="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R17="禁发",S17="禁发",T17="禁发"),"禁发",IF(AND(R17="资料确认",S17="通过",T17="通过"),"资料参数可发布",IF(AND(R17="行业推定",S17="通过",T17="通过"),"范围表达可发布",IF(AND(R17="通过",S17="通过",T17="通过"),"精确值可发布",IF(AND(S17="通过",R17="待唐工复核",T17="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V17" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W17" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W17" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X17" s="25" t="str">
-        <x:v>资料中出现服务响应和固定周期类表述，公开前需全部降级为合同约定。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F19：F19 核心参数资料确认，工艺曲线与组织指标为行业推定。改造案例不新建页面，等待 UI 审核门。</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -19306,7 +19293,7 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I18" s="25" t="str">
-        <x:v>资料中出现炉膛尺寸约 13×7.4×4.3m，额定温度 700℃，14 套燃气烧嘴，助燃空气预热约 250-300℃；公开时避免节能率承诺。</x:v>
+        <x:v>超大型台车炉有效加热区 13×7.4×4.3 m；额定/最高使用温度 700℃；原电阻炉改为天然气燃气炉。按 14 个温控区及 14×630 kW=8820 kW 核对，方案采用 14 套 630 kW 级高速天然气烧嘴；助燃空气 250–300℃为设计目标。</x:v>
       </x:c>
       <x:c r="J18" s="25" t="str">
         <x:v>原电阻炉改燃气、超大炉膛密封、炉压控制、烧嘴布置、余热回收和安全联锁。</x:v>
@@ -19315,13 +19302,13 @@
         <x:v>电改燃方案、燃烧系统、密封改造、炉压与排烟余热回收、控制系统升级。</x:v>
       </x:c>
       <x:c r="L18" s="25" t="str">
-        <x:v>可作为工业炉节能改造与台车炉改造项目经验模块。</x:v>
+        <x:v>有效尺寸、温度、能源改造方向和 14 区/8820 kW 方案口径可发布；烧嘴布置只能作为设计推定，不写品牌型号。</x:v>
       </x:c>
       <x:c r="M18" s="25" t="str">
-        <x:v>客户全称、节能率/热效率绝对承诺、燃气管路图、报价和付款条款。</x:v>
+        <x:v>不得采用旧模板“10 套烧嘴”；不得编造烧嘴品牌型号；不得把两侧各 7 套或 250–300℃写成实测验收结果。</x:v>
       </x:c>
       <x:c r="N18" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-014</x:v>
+        <x:v>100_样本_节能燃气式台车式退火炉改造_技术方案_2020.pdf</x:v>
       </x:c>
       <x:c r="O18" s="25" t="str">
         <x:v>是</x:v>
@@ -19333,7 +19320,7 @@
         <x:v>台车炉现有产品页</x:v>
       </x:c>
       <x:c r="R18" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S18" s="25" t="str">
         <x:v>通过</x:v>
@@ -19342,18 +19329,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U18" s="25" t="str">
-        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(AND(S18="通过",R18="待唐工复核",T18="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R18="禁发",S18="禁发",T18="禁发"),"禁发",IF(AND(R18="资料确认",S18="通过",T18="通过"),"资料参数可发布",IF(AND(R18="行业推定",S18="通过",T18="通过"),"范围表达可发布",IF(AND(R18="通过",S18="通过",T18="通过"),"精确值可发布",IF(AND(S18="通过",R18="待唐工复核",T18="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V18" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W18" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W18" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X18" s="25" t="str">
-        <x:v>公开时要删除“同行领先”等风险表述，只保留按工况评估。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F20：F20 核心参数资料确认，具体布置为行业推定。官网使用“630 kW 级高速天然气烧嘴”。</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -19382,7 +19368,7 @@
         <x:v>新建 / 单炉设备</x:v>
       </x:c>
       <x:c r="I19" s="25" t="str">
-        <x:v>资料中出现 REWF-45-9 型，网带尺寸约 2100×200×50mm，有效宽度约 180mm，额定温度 950℃，产量约 60kg/h，网带速度约 10-114mm/min。</x:v>
+        <x:v>REWF-45-9 马弗式保护气氛电加热网带炉：额定功率 45 kW、额定/最高工作温度约 950℃；加热长度 2100 mm、名义网带宽 200 mm、有效工作宽 180 mm、有效装料高度 50 mm；网带速度 10–114 mm/min；理论停留时间约 18.4–210 min。最大设计能力约 60 kg/h，计算为 0.18×0.114×60×50=61.56 kg/h。</x:v>
       </x:c>
       <x:c r="J19" s="25" t="str">
         <x:v>小型工件保护气氛、马弗罐密封、网带传动和活动料框出料、淬火油槽温度控制。</x:v>
@@ -19391,13 +19377,13 @@
         <x:v>马弗式保护气氛网带炉、淬火油槽、气氛和温控系统。</x:v>
       </x:c>
       <x:c r="L19" s="25" t="str">
-        <x:v>可用于网带炉页面项目经验，说明保护气氛网带炉配置能力。</x:v>
+        <x:v>尺寸、速度和带计算条件的最大设计能力可发布；实际产量按工件、铺料和加热时间确定。</x:v>
       </x:c>
       <x:c r="M19" s="25" t="str">
-        <x:v>客户全称、工件具体型号、气氛配方细节、验收条款和报价。</x:v>
+        <x:v>不得把 60 kg/h 写成实际验收产量；不得脱离最大速度和 50 kg/㎡面载荷引用该数字。</x:v>
       </x:c>
       <x:c r="N19" s="25" t="str">
-        <x:v>docs/seo-geo/case-assets-dedup.json#SN-CASE-P1-015</x:v>
+        <x:v>100_样本_马弗式保护气氛网带炉_技术方案_20201114.pdf</x:v>
       </x:c>
       <x:c r="O19" s="25" t="str">
         <x:v>是</x:v>
@@ -19409,7 +19395,7 @@
         <x:v>网带炉现有产品页</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
         <x:v>通过</x:v>
@@ -19418,18 +19404,17 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(AND(S19="通过",R19="待唐工复核",T19="通过"),"公开（技术复核待完成）","待审核")))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:f>IF(OR(R19="禁发",S19="禁发",T19="禁发"),"禁发",IF(AND(R19="资料确认",S19="通过",T19="通过"),"资料参数可发布",IF(AND(R19="行业推定",S19="通过",T19="通过"),"范围表达可发布",IF(AND(R19="通过",S19="通过",T19="通过"),"精确值可发布",IF(AND(S19="通过",R19="待唐工复核",T19="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V19" s="25" t="str">
-        <x:v>待安排：唐登荣</x:v>
-      </x:c>
-      <x:c r="W19" s="26"/>
+        <x:v>资料依据核对（非个人 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W19" s="26" t="n">
+        <x:v>46232</x:v>
+      </x:c>
       <x:c r="X19" s="25" t="str">
-        <x:v>更适合产品页补充，不建议单独案例页。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>F21：F21 资料确认。公式、单位与适用条件必须和设计能力同页呈现。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -19494,7 +19479,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U20" s="25" t="str">
-        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(AND(S20="通过",R20="待唐工复核",T20="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R20="禁发",S20="禁发",T20="禁发"),"禁发",IF(AND(R20="资料确认",S20="通过",T20="通过"),"资料参数可发布",IF(AND(R20="行业推定",S20="通过",T20="通过"),"范围表达可发布",IF(AND(R20="通过",S20="通过",T20="通过"),"精确值可发布",IF(AND(S20="通过",R20="待唐工复核",T20="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V20" s="25"/>
@@ -19567,7 +19552,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U21" s="25" t="str">
-        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(AND(S21="通过",R21="待唐工复核",T21="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R21="禁发",S21="禁发",T21="禁发"),"禁发",IF(AND(R21="资料确认",S21="通过",T21="通过"),"资料参数可发布",IF(AND(R21="行业推定",S21="通过",T21="通过"),"范围表达可发布",IF(AND(R21="通过",S21="通过",T21="通过"),"精确值可发布",IF(AND(S21="通过",R21="待唐工复核",T21="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V21" s="25"/>
@@ -19640,7 +19625,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U22" s="25" t="str">
-        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(AND(S22="通过",R22="待唐工复核",T22="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R22="禁发",S22="禁发",T22="禁发"),"禁发",IF(AND(R22="资料确认",S22="通过",T22="通过"),"资料参数可发布",IF(AND(R22="行业推定",S22="通过",T22="通过"),"范围表达可发布",IF(AND(R22="通过",S22="通过",T22="通过"),"精确值可发布",IF(AND(S22="通过",R22="待唐工复核",T22="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>禁发</x:v>
       </x:c>
       <x:c r="V22" s="25"/>
@@ -19713,7 +19698,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U23" t="str">
-        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",R23="待唐工复核",T23="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="资料确认",S23="通过",T23="通过"),"资料参数可发布",IF(AND(R23="行业推定",S23="通过",T23="通过"),"范围表达可发布",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",R23="待唐工复核",T23="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V23" t="str">
@@ -19789,7 +19774,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U24" t="str">
-        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(AND(S24="通过",R24="待唐工复核",T24="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R24="禁发",S24="禁发",T24="禁发"),"禁发",IF(AND(R24="资料确认",S24="通过",T24="通过"),"资料参数可发布",IF(AND(R24="行业推定",S24="通过",T24="通过"),"范围表达可发布",IF(AND(R24="通过",S24="通过",T24="通过"),"精确值可发布",IF(AND(S24="通过",R24="待唐工复核",T24="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V24" t="str">
@@ -19865,7 +19850,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U25" t="str">
-        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(AND(S25="通过",R25="待唐工复核",T25="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R25="禁发",S25="禁发",T25="禁发"),"禁发",IF(AND(R25="资料确认",S25="通过",T25="通过"),"资料参数可发布",IF(AND(R25="行业推定",S25="通过",T25="通过"),"范围表达可发布",IF(AND(R25="通过",S25="通过",T25="通过"),"精确值可发布",IF(AND(S25="通过",R25="待唐工复核",T25="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V25" t="str">
@@ -19941,7 +19926,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U26" t="str">
-        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(AND(S26="通过",R26="待唐工复核",T26="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R26="禁发",S26="禁发",T26="禁发"),"禁发",IF(AND(R26="资料确认",S26="通过",T26="通过"),"资料参数可发布",IF(AND(R26="行业推定",S26="通过",T26="通过"),"范围表达可发布",IF(AND(R26="通过",S26="通过",T26="通过"),"精确值可发布",IF(AND(S26="通过",R26="待唐工复核",T26="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V26" t="str">
@@ -20017,7 +20002,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U27" t="str">
-        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",R27="待唐工复核",T27="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="资料确认",S27="通过",T27="通过"),"资料参数可发布",IF(AND(R27="行业推定",S27="通过",T27="通过"),"范围表达可发布",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",R27="待唐工复核",T27="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V27" t="str">
@@ -20093,7 +20078,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="U28" t="str">
-        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(AND(S28="通过",R28="待唐工复核",T28="通过"),"公开（技术复核待完成）","待审核")))</x:f>
+        <x:f>IF(OR(R28="禁发",S28="禁发",T28="禁发"),"禁发",IF(AND(R28="资料确认",S28="通过",T28="通过"),"资料参数可发布",IF(AND(R28="行业推定",S28="通过",T28="通过"),"范围表达可发布",IF(AND(R28="通过",S28="通过",T28="通过"),"精确值可发布",IF(AND(S28="通过",R28="待唐工复核",T28="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V28" t="str">
@@ -20114,7 +20099,7 @@
   <x:conditionalFormatting sqref="U5:U22">
     <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="待审核"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="5">
+  <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="R5:T22">
       <x:formula1>"待确认,通过,范围表达,禁发"</x:formula1>
     </x:dataValidation>
@@ -20130,10 +20115,16 @@
     <x:dataValidation type="list" sqref="R5:T28">
       <x:formula1>"待确认,通过,范围表达,禁发,待唐工复核"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="R5:R28">
+      <x:formula1>"资料确认,行业推定,待唐工复核,待确认,通过,禁发"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="S5:T28">
+      <x:formula1>"待确认,通过,范围表达,禁发"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a2b234ea0214cf5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R832b6445365e4818"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20520,6 +20511,61 @@
         <x:v>提交成功只代表收到；继续用 nginx 日志检查实际抓取</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" t="str">
+        <x:v>技术状态</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>资料确认</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>现有方案、报价、合同台账或证书有明确依据；可按项目级设计参数发布</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" t="str">
+        <x:v>技术状态</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>行业推定</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>由炉型、功率、尺寸、速度或工艺推算；只能写典型工况、设计目标或通常配置</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" t="str">
+        <x:v>发布状态</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>资料参数可发布</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>资料来源明确且公司、客户范围允许；仍须保留项目条件，不代表验收实绩</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>发布状态</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>范围表达可发布</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>只能使用典型、通常、设计目标等范围措辞，不发布为项目实测结果</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" t="str">
+        <x:v>禁止口径</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>禁止写成实绩</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>缺验收、检测或个人授权时，不写实测、实际产量、已验收、正式职称或 reviewedBy</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F2"/>

</xml_diff>

<commit_message>
feat(geo): publish second authority topic batch
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R5d9647bc12b74606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R8dc84fa6b42441b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R95f407890feb4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R64c2787391994e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Raf7ef506169a4b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="Rba30bae2792e467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R457a0e980ebb44c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R4b8f8fce770c44b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R40b9765d724247b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="R25019c569b7f47d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -114,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -181,6 +181,7 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -798,15 +799,13 @@
         <x:v>事实资产发布状态</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"资料参数可发布")+COUNTIF('事实单元'!$U$5:$U$28,"范围表达可发布")+COUNTIF('事实单元'!$U$5:$U$28,"精确值可发布")</x:f>
-        <x:v>15</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:f>COUNTIF('事实单元'!$U$5:$U$28,"资料参数可发布")&amp;" 项资料参数可发布；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"公开（技术复核待完成）")&amp;" 项高责任事实待补；"&amp;COUNTIF('事实单元'!$U$5:$U$28,"禁发")&amp;" 项禁发"</x:f>
-        <x:v>15 项资料参数可发布；6 项高责任事实待补；3 项禁发</x:v>
+        <x:v>21 项可发布（15 项资料参数 + 6 项 P5 技术方法）</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>F07–F21 已按资料确认、行业推定和禁止实绩三层口径完成分级；青山经济测算、项目周期与排放结论仍按独立高责任事实管理，资料未齐前不升级为验收实绩。</x:v>
+        <x:v>新增 Q1–Q6 技术方法事实已按钱波提供的最终答复完成确认；青山经济测算、项目周期与排放结论仍按独立高责任事实管理，资料未齐前不升级。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16142,7 +16141,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re872a5316df14077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3cf37a6137b4009"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18126,7 +18125,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d256f9e193e4b4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1666b2887594c97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18163,7 +18162,7 @@
   <x:sheetData>
     <x:row r="1" ht="54" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>苏能 GEO 事实单元与三门审核台账（18 项案例资产 + 6 项高风险事实）</x:v>
+        <x:v>苏能 GEO 事实单元与三门审核台账（18 项案例资产 + 6 项高风险事实 + 6 项 P5 技术方法事实）</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -18191,8 +18190,8 @@
     </x:row>
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>24 项事实单元与三门审核
-21 项授权状态已确认，唐登荣技术复核待完成；3 项 P2 弱相关资料继续禁发。现有页面可以保留，技术复核完成前不得新增未经复核的精确值、跨页复用或站外分发。</x:v>
+        <x:v>30 项事实单元与三门审核
+15 项资料参数、6 项 P5 技术方法可发布；6 项青山高责任事实仍待底稿复核；3 项 P2 弱相关资料继续禁发。P5 技术方法可以按确认边界用于 C/D 权威主题页，但不得写成具体项目实际安装、实测或验收结果。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -18364,7 +18363,7 @@
         <x:v>46232</x:v>
       </x:c>
       <x:c r="X5" s="25" t="str">
-        <x:v>F07：F07 资料确认。PC200–PC400 为工件型号范围；950℃为额定温度，不是实际淬火工艺温度。资料确认不等于个人 reviewedBy，当前不启用唐登荣复核身份。</x:v>
+        <x:v>F07：F07 资料确认。PC200–PC400 为工件型号范围；950℃为额定温度，不是实际淬火工艺温度。资料确认不等于个人 reviewedBy，当前不启用唐工复核身份。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -19665,16 +19664,16 @@
         <x:v>产线数量、宽度和改造规模：原页面写为 3 条 1250mm 连续退洗线。</x:v>
       </x:c>
       <x:c r="J23" t="str">
-        <x:v>项目规模属于客户与合同边界信息；必须确认是否为同一项目、同一改造批次，并取得公开范围授权。</x:v>
+        <x:v>项目规模属于客户与合同边界信息；技术上必须确认是否为同一项目、同一改造批次，公开范围按已授权口径执行。</x:v>
       </x:c>
       <x:c r="K23" t="str">
         <x:v>核对合同/技术协议、总图或设备清单，确认可公开的数量与规格口径。</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>可公开为“多条连续退洗线节能改造”，具体规格与数量待授权确认。</x:v>
+        <x:v>可公开为“多条连续退洗线节能改造”，具体规格与数量待唐工复核确认。</x:v>
       </x:c>
       <x:c r="M23" t="str">
-        <x:v>未核实或未授权前，不公开“3 条”“1250mm”及其组合，不用客户集团线索反推主体。</x:v>
+        <x:v>唐工完成技术复核前，不公开“3 条”“1250mm”及其组合；不用客户集团线索反推主体。</x:v>
       </x:c>
       <x:c r="N23" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -19702,14 +19701,14 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V23" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W23"/>
       <x:c r="X23" t="str">
         <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19750,7 +19749,7 @@
         <x:v>可公开为“具备降低综合能耗成本的空间，实际收益需按项目工况测算”。</x:v>
       </x:c>
       <x:c r="M24" t="str">
-        <x:v>三门未全过前不公开 7,644 万元/年，不把测算值写成客户实际收益或通用承诺。</x:v>
+        <x:v>唐工完成技术复核前，不公开 7,644 万元/年，不把测算值写成客户实际收益或通用承诺。</x:v>
       </x:c>
       <x:c r="N24" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -19778,14 +19777,14 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V24" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W24"/>
       <x:c r="X24" t="str">
         <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -19826,7 +19825,7 @@
         <x:v>可公开为“单位产品能耗成本具备下降空间，幅度按现场数据单独核算”。</x:v>
       </x:c>
       <x:c r="M25" t="str">
-        <x:v>三门未全过前不公开 63.7 元/吨，不与任何未核年产量拼接成收益公式。</x:v>
+        <x:v>唐工完成技术复核前，不公开 63.7 元/吨，不与任何未核年产量拼接成收益公式。</x:v>
       </x:c>
       <x:c r="N25" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -19854,14 +19853,14 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V25" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W25"/>
       <x:c r="X25" t="str">
         <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19902,7 +19901,7 @@
         <x:v>可公开为“收益测算需使用经双方确认的有效产量或运行负荷”。</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>三门未全过前不公开 120 万吨/年，不将测算分母描述为客户实际产能或经营数据。</x:v>
+        <x:v>唐工完成技术复核前，不公开 120 万吨/年，不将测算分母描述为客户实际产能或经营数据。</x:v>
       </x:c>
       <x:c r="N26" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -19930,14 +19929,14 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V26" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W26"/>
       <x:c r="X26" t="str">
         <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -19978,7 +19977,7 @@
         <x:v>可公开为“各阶段周期按项目规模、供货边界和停产窗口在合同中确认”。</x:v>
       </x:c>
       <x:c r="M27" t="str">
-        <x:v>没有完整里程碑证据前，不公开固定设计、制造、安装或验收周期。</x:v>
+        <x:v>唐工完成技术复核且取得完整里程碑证据前，不公开固定设计、制造、安装或验收周期。</x:v>
       </x:c>
       <x:c r="N27" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -20006,14 +20005,14 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V27" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W27"/>
       <x:c r="X27" t="str">
         <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20054,7 +20053,7 @@
         <x:v>可公开为“按所在地排放要求设计，是否达标以有资质第三方检测或正式验收为准”。</x:v>
       </x:c>
       <x:c r="M28" t="str">
-        <x:v>未取得可核验报告及授权前，不写“已达标”“满足国家标准”或具体排放数值。</x:v>
+        <x:v>未取得可核验报告并完成唐工技术复核前，不写“已达标”“满足国家标准”或具体排放数值。</x:v>
       </x:c>
       <x:c r="N28" t="str">
         <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
@@ -20082,14 +20081,464 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="V28" t="str">
-        <x:v>待安排：唐登荣</x:v>
+        <x:v>待安排：唐工</x:v>
       </x:c>
       <x:c r="W28"/>
       <x:c r="X28" t="str">
         <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。
 2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐登荣技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐登荣技术签审，公开时必须保留项目级适用边界。</x:v>
+GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
+2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>SN-GEO-P5-CD-Q01</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>炉衬局部修复、扩大拆检与整体处理判断</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>炉衬与保温</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>技术方法</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>不使用通用面积比例；以支撑体系、冷面状态、锚固连续性、失效原因和接缝条件综合判断。</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>局部损坏、冷面完好、区外锚固完好、原因局部且新旧衬可可靠衔接时可考虑局部修复；炉顶下沉、冷面异常升温、贯通裂缝等应扩大拆检。</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>停炉检查、开衬复核、炉衬方案核算和修复范围确认。</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>炉衬是否局部修复，不能只看热面损坏面积；应同时检查冷面钢板、锚固体系、失效原因和新旧衬接缝条件。出现炉顶下沉、冷面异常升温或贯通裂缝等信号时，应扩大拆检，最终范围以停炉检查为准。</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>不得把风险信号写成脱离检查条件的绝对否决项；改燃料、升温、增加装炉量时不得直接沿用旧炉衬结论。</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>2020 台车炉电改燃方案第 5 页；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q29" t="str">
+        <x:v>P5 C 页：炉衬翻新与保温</x:v>
+      </x:c>
+      <x:c r="R29" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S29" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T29" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U29" t="str">
+        <x:f>IF(OR(R29="禁发",S29="禁发",T29="禁发"),"禁发",IF(AND(R29="资料确认",S29="通过",T29="通过"),"资料参数可发布",IF(AND(R29="行业推定",S29="通过",T29="通过"),"范围表达可发布",IF(AND(R29="通过",S29="通过",T29="通过"),"精确值可发布",IF(AND(S29="通过",R29="待唐工复核",T29="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V29" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W29" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X29" t="str">
+        <x:v>Q1 已确认。可作为采购判断方法复用；具体项目范围仍需停炉检查。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>SN-GEO-P5-CD-Q02</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>1140 型纤维模块与压缩量≥40%的事实边界</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>纤维炉衬</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>方案参数解释</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>2018 项目技术方案载明“1140 型耐火纤维模块、压缩量≥40%”；只能确认为项目方案参数。</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>压缩量反映预补偿高温收缩、维持模块接缝压紧的设计意图；准确计算基准和适用性取决于材料、模块结构与安装方向。</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>材料牌号核对、产品合格证核对、施工方案与安装记录确认。</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>某项目技术方案采用“1140 型耐火纤维模块、压缩量≥40%”的设计参数；具体牌号含义和安装压缩要求，应结合产品合格证、材料体系与施工方案确认。</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>不得推断 1140 型的分类温度；不得把≥40%写成所有炉型通用标准；不得发布无记录支撑的寿命时间结论。</x:v>
+      </x:c>
+      <x:c r="N30" t="str">
+        <x:v>2018 两用型改造技术方案第 5 页及参数表；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O30" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q30" t="str">
+        <x:v>P5 C 页：炉衬翻新与保温</x:v>
+      </x:c>
+      <x:c r="R30" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S30" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T30" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U30" t="str">
+        <x:f>IF(OR(R30="禁发",S30="禁发",T30="禁发"),"禁发",IF(AND(R30="资料确认",S30="通过",T30="通过"),"资料参数可发布",IF(AND(R30="行业推定",S30="通过",T30="通过"),"范围表达可发布",IF(AND(R30="通过",S30="通过",T30="通过"),"精确值可发布",IF(AND(S30="通过",R30="待唐工复核",T30="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V30" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W30" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X30" t="str">
+        <x:v>Q2 已确认。鲁阳历史产品资料、合格证和施工记录仍待调取；不影响发布当前边界表达。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>SN-GEO-P5-CD-Q03</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>烘炉制度、责任边界与交付记录</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>耐材施工与烘炉</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>技术方法</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>不发布统一温度平台、升温速度或固定时长。</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>烘炉制度由材料边界、耐材组合、施工厚度、含水情况、排湿条件、环境与炉型共同决定；不同耐材体系不可直接套用同一曲线。</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>烘炉制度编制、执行记录、排湿观察和异常闭环。</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>烘炉曲线应由耐材体系、施工厚度、含水情况、排湿条件和炉型共同决定；验收应看实测曲线、排汽和异常记录，不能只以“烘了多少小时”作为完成依据。</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>不得发布跨材料体系的通用烘炉曲线；不得用固定小时数单独判定水分排出完成。</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>本机未检出可跨项目复用的完整烘炉曲线；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q31" t="str">
+        <x:v>P5 C 页：炉衬翻新与保温</x:v>
+      </x:c>
+      <x:c r="R31" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S31" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T31" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U31" t="str">
+        <x:f>IF(OR(R31="禁发",S31="禁发",T31="禁发"),"禁发",IF(AND(R31="资料确认",S31="通过",T31="通过"),"资料参数可发布",IF(AND(R31="行业推定",S31="通过",T31="通过"),"范围表达可发布",IF(AND(R31="通过",S31="通过",T31="通过"),"精确值可发布",IF(AND(S31="通过",R31="待唐工复核",T31="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V31" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W31" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X31" t="str">
+        <x:v>Q3 已确认。交付记录至少包含实测曲线、保温时长、排湿口状态、排汽观察、异常处理和环境温湿度。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>SN-GEO-P5-CD-Q04</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>燃气安全功能与 FAT/SAT 证据边界</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>燃气燃烧与安全</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>技术方法</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>不设置脱离炉型、燃料、风险等级与属地规范的统一配置数量。</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>安全链通常围绕吹扫、程序点火、火焰检测与失焰切断、燃气压力、助燃风、停电失效安全、紧急切断、阀组隔离和泄漏报警设计。</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>FAT 控制逻辑与动作验证；SAT 现场管路、真实工况和联锁验证。</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>FAT 主要证明控制逻辑和安全动作按设计工作，SAT 还要证明这台炉、这套管路和现场燃气条件下能够安全运行；FAT 不能替代 SAT。</x:v>
+      </x:c>
+      <x:c r="M32" t="str">
+        <x:v>不得把旧技术方案未枚举的电气细节解释为未配置；不得把补充清单写成所有项目完全相同的最低配置。</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
+        <x:v>相关燃气改造技术方案文本；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O32" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P32" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q32" t="str">
+        <x:v>P5 D 页：电改燃与余热回收</x:v>
+      </x:c>
+      <x:c r="R32" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S32" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T32" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U32" t="str">
+        <x:f>IF(OR(R32="禁发",S32="禁发",T32="禁发"),"禁发",IF(AND(R32="资料确认",S32="通过",T32="通过"),"资料参数可发布",IF(AND(R32="行业推定",S32="通过",T32="通过"),"范围表达可发布",IF(AND(R32="通过",S32="通过",T32="通过"),"精确值可发布",IF(AND(S32="通过",R32="待唐工复核",T32="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V32" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W32" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X32" t="str">
+        <x:v>Q4 已确认。标准号与版本须按具体项目和属地规范核对后再引用。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>SN-GEO-P5-CD-Q05</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>两用燃料的燃料侧隔离与切换顺序</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>两用燃料系统</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>技术方法</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>2018 方案只确认助燃空气支路换向；不能由断风推导燃料侧已隔离。</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>切换应围绕当前燃料停火、燃料侧切断及阀位反馈、炉膛吹扫、系统切换、目标燃料条件确认和完整重新点火组织。</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>燃料管路、电气图、PLC 点表、模式互锁和现场验证。</x:v>
+      </x:c>
+      <x:c r="L33" t="str">
+        <x:v>两用燃料切换的核心是燃料侧切断、实际阀位反馈、模式互锁和吹扫完成共同构成点火许可；空气侧断风不能替代燃料侧安全隔离。</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>不得写成 2018 项目已经安装或验收了燃料侧隔离；不得由关闭燃油烧嘴供风推断两种燃料不可能同时供入。</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>2018 两用型改造技术方案；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O33" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q33" t="str">
+        <x:v>P5 D 页：电改燃与余热回收</x:v>
+      </x:c>
+      <x:c r="R33" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S33" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T33" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U33" t="str">
+        <x:f>IF(OR(R33="禁发",S33="禁发",T33="禁发"),"禁发",IF(AND(R33="资料确认",S33="通过",T33="通过"),"资料参数可发布",IF(AND(R33="行业推定",S33="通过",T33="通过"),"范围表达可发布",IF(AND(R33="通过",S33="通过",T33="通过"),"精确值可发布",IF(AND(S33="通过",R33="待唐工复核",T33="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V33" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W33" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X33" t="str">
+        <x:v>Q5 已确认。具体项目实际配置仍需电气图、燃油管路图、PLC 点表或竣工资料。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>SN-GEO-P5-CD-Q06</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>炉体外表面温升指标转化为验收条件</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>不涉及客户身份</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>通用方法</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>工业炉改造</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>炉衬与保温验收</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>设计指标与验收方法</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>2018 项目技术方案设计边界：使用温度 800℃、达到稳定态、热桥除外时，炉体外表面温升不超过 40 K。</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>若转成验收条件，必须约定测点、热桥排除、稳定态判定、环境温度取值、测量仪器及红外发射率。</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>技术协议测量规则、现场测温记录和验收资料核对。</x:v>
+      </x:c>
+      <x:c r="L34" t="str">
+        <x:v>某项目技术方案采用“炉子使用温度 800℃、达到稳定态、热桥除外时，炉体外表面温升不超过 40 K”的设计指标；如用于验收，还需在技术协议中明确测点、稳定态、环境温度、仪器与热桥排除规则。</x:v>
+      </x:c>
+      <x:c r="M34" t="str">
+        <x:v>不得外推成所有炉型通用承诺；无现场记录时不得写成客户验收结果或实测值。</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>2018 两用型改造技术方案技术参数表第 17 项；docs/seo-geo/p5-cd-tang-confirmation-checklist.md（2026-07-31 钱波提供最终技术答复）</x:v>
+      </x:c>
+      <x:c r="O34" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="P34" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="Q34" t="str">
+        <x:v>P5 C 页：炉衬翻新与保温</x:v>
+      </x:c>
+      <x:c r="R34" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="S34" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="T34" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="U34" t="str">
+        <x:f>IF(OR(R34="禁发",S34="禁发",T34="禁发"),"禁发",IF(AND(R34="资料确认",S34="通过",T34="通过"),"资料参数可发布",IF(AND(R34="行业推定",S34="通过",T34="通过"),"范围表达可发布",IF(AND(R34="通过",S34="通过",T34="通过"),"精确值可发布",IF(AND(S34="通过",R34="待唐工复核",T34="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
+        <x:v>精确值可发布</x:v>
+      </x:c>
+      <x:c r="V34" t="str">
+        <x:v>唐工答复（由钱波转交；非 reviewedBy）</x:v>
+      </x:c>
+      <x:c r="W34" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="X34" t="str">
+        <x:v>Q6 已确认。当前发布的是项目设计指标与验收方法，不是现场实测结果。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20124,7 +20573,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R832b6445365e4818"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R739ffce751c6460f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20231,7 +20680,7 @@
       </x:c>
       <x:c r="D5" s="29"/>
       <x:c r="E5" s="17" t="str">
-        <x:v>唐登荣</x:v>
+        <x:v>唐工</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
         <x:v>技术准确、适用边界、工程事实复核</x:v>
@@ -20447,14 +20896,14 @@
         <x:v>待唐工复核</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>只完成行业常识初筛，尚未取得唐登荣本人技术复核记录</x:v>
+        <x:v>只完成行业常识初筛，尚未取得唐工本人技术复核记录</x:v>
       </x:c>
       <x:c r="D19"/>
       <x:c r="E19" t="str">
         <x:v>录音转写</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>经唐登荣知情同意后录音；本人只回答和确认，整理工作后置</x:v>
+        <x:v>经唐工知情同意后录音；本人只回答和确认，整理工作后置</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -20483,7 +20932,7 @@
         <x:v>公开（技术复核待完成）</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>现有页面可保留；唐登荣技术复核完成前，不新增未经复核的精确值、跨页复用或站外分发</x:v>
+        <x:v>现有页面可保留；唐工技术复核完成前，不新增未经复核的精确值、跨页复用或站外分发</x:v>
       </x:c>
       <x:c r="D21"/>
       <x:c r="E21" t="str">

</xml_diff>

<commit_message>
docs(geo): close P1 evidence and monitoring
</commit_message>
<xml_diff>
--- a/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
+++ b/docs/seo-geo/苏能GEO监测与事实台账_2026-07-29.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="Rba30bae2792e467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R457a0e980ebb44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R4b8f8fce770c44b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R40b9765d724247b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="R25019c569b7f47d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基线总览" sheetId="1" r:id="R1c814d24b1714b55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="复测明细" sheetId="2" r:id="R08f38ab7967a4017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55问题库" sheetId="3" r:id="R7221fed9fa1c43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事实单元" sheetId="4" r:id="R27b64918fed64f63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核字典" sheetId="5" r:id="Rf51783ffc25b401c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -794,18 +794,18 @@
       <x:c r="G10" s="21"/>
       <x:c r="H10" s="21"/>
     </x:row>
-    <x:row r="11" ht="46.5" customHeight="1">
+    <x:row r="11" ht="88.5" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>事实资产发布状态</x:v>
       </x:c>
       <x:c r="B11" s="19" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>21 项可发布（15 项资料参数 + 6 项 P5 技术方法）</x:v>
+        <x:v>23 项可发布（17 项资料参数 + 6 项 P5 技术方法）</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>新增 Q1–Q6 技术方法事实已按钱波提供的最终答复完成确认；青山经济测算、项目周期与排放结论仍按独立高责任事实管理，资料未齐前不升级。</x:v>
+        <x:v>新增 Q1–Q6 技术方法事实已按钱波提供的最终答复完成确认；青山 F01 与 F05 已完成合同/技术方案原件核查并升级为资料确认。F02–F04 仍是技术方案测算值，F06 缺第三方检测/验收报告，继续按独立高责任事实管理。</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
         <x:v>复测决策门</x:v>
@@ -16141,7 +16141,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3cf37a6137b4009"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd46120f844284ed0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18125,7 +18125,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1666b2887594c97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00edbb87fb1e43ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19661,22 +19661,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I23" t="str">
-        <x:v>产线数量、宽度和改造规模：原页面写为 3 条 1250mm 连续退洗线。</x:v>
+        <x:v>一期1250mm连续退洗线（三条线）；1250mm为机组名义规格及方案最大带宽，方案产品宽度范围为800～1250mm。</x:v>
       </x:c>
       <x:c r="J23" t="str">
-        <x:v>项目规模属于客户与合同边界信息；技术上必须确认是否为同一项目、同一改造批次，公开范围按已授权口径执行。</x:v>
+        <x:v>3条线和1250mm由同一项目合同与技术方案直接确认；实际运行带宽仍取决于产品规格。</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>核对合同/技术协议、总图或设备清单，确认可公开的数量与规格口径。</x:v>
+        <x:v>合同/技术方案资料核对，确认项目数量、名义规格和产品宽度边界。</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>可公开为“多条连续退洗线节能改造”，具体规格与数量待唐工复核确认。</x:v>
+        <x:v>一期1250mm连续退洗线三线改造；1250mm为机组名义规格和本方案最大带宽，实际处理带宽范围为800～1250mm。</x:v>
       </x:c>
       <x:c r="M23" t="str">
-        <x:v>唐工完成技术复核前，不公开“3 条”“1250mm”及其组合；不用客户集团线索反推主体。</x:v>
+        <x:v>不得把1250mm写成所有工况下的固定实际带宽；不得跨项目套用数量和规格；不得用脱敏线索反推客户主体。</x:v>
       </x:c>
       <x:c r="N23" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>主合同第2页“项目内容及配置清单”：一期1250mm连续退洗线（三条线），规格DXKJ-1250-GZ；本项目技术方案“一、项目内容”数量3线及“产品规格”B=800～1250mm。</x:v>
       </x:c>
       <x:c r="O23" t="str">
         <x:v>是</x:v>
@@ -19688,7 +19688,7 @@
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R23" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S23" t="str">
         <x:v>通过</x:v>
@@ -19698,17 +19698,16 @@
       </x:c>
       <x:c r="U23" t="str">
         <x:f>IF(OR(R23="禁发",S23="禁发",T23="禁发"),"禁发",IF(AND(R23="资料确认",S23="通过",T23="通过"),"资料参数可发布",IF(AND(R23="行业推定",S23="通过",T23="通过"),"范围表达可发布",IF(AND(R23="通过",S23="通过",T23="通过"),"精确值可发布",IF(AND(S23="通过",R23="待唐工复核",T23="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V23" t="str">
-        <x:v>待安排：唐工</x:v>
-      </x:c>
-      <x:c r="W23"/>
+        <x:v>合同/技术方案资料核对</x:v>
+      </x:c>
+      <x:c r="W23" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
       <x:c r="X23" t="str">
-        <x:v>所需证据：合同或技术附件、总图/设备清单、公司公开批准、客户授权记录。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：主合同第2页及本项目技术方案直接写明3线、1250mm；参数表给出B=800～1250mm。可按项目规格发布，必须保留宽度边界；不等于长期运行记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -19737,22 +19736,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I24" t="str">
-        <x:v>年节能效益：原页面写为约 7,644 万元/年。</x:v>
+        <x:v>2015年技术方案测算值：7,644万元/年=(117-53.3)元/吨×120万吨/年。</x:v>
       </x:c>
       <x:c r="J24" t="str">
-        <x:v>收益受燃料价格、负荷、运行天数、改造边界和统计区间影响，属于高责任经济性结论。</x:v>
+        <x:v>方案以天然气改冷煤气、能源价格和三条线年产量假设进行经济性测算；不是客户实际财务结果或验收结果。</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>复核改造前后原始能耗与产量台账、计算表、价格口径和统计区间。</x:v>
+        <x:v>复核方案计算公式；后续仍需改造前后同工况能耗台账、实际能源价格、税口径和客户确认痕迹。</x:v>
       </x:c>
       <x:c r="L24" t="str">
-        <x:v>可公开为“具备降低综合能耗成本的空间，实际收益需按项目工况测算”。</x:v>
+        <x:v>2015年技术方案按当时能源价格和三条线年产量假设测算，年燃料成本差额约7,644万元；仅适用于本项目方案测算，不代表实际收益。</x:v>
       </x:c>
       <x:c r="M24" t="str">
-        <x:v>唐工完成技术复核前，不公开 7,644 万元/年，不把测算值写成客户实际收益或通用承诺。</x:v>
+        <x:v>不得写成客户实际收益、验收结果或通用节能承诺；唐工复核前不得跨页面或站外复用。</x:v>
       </x:c>
       <x:c r="N24" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>本项目技术方案“三、项目说明—A、经济性分析”：天然气117元/吨、冷煤气53.3元/吨，三条线按年产量120万吨计算，(117-53.3)×120万吨=7644万元。未检出实际能耗/财务验收底稿。</x:v>
       </x:c>
       <x:c r="O24" t="str">
         <x:v>是</x:v>
@@ -19779,12 +19778,9 @@
       <x:c r="V24" t="str">
         <x:v>待安排：唐工</x:v>
       </x:c>
-      <x:c r="W24"/>
+      <x:c r="W24" s="30"/>
       <x:c r="X24" t="str">
-        <x:v>所需证据：原始能耗/产量记录、节能测算底稿、燃料价格边界、运行制度、技术审核、公司批准、客户授权。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：测算公式有技术方案出处，但未检出实际能耗/财务验收底稿，也未明确基准期、测算期和税口径。当前只能标为方案测算，不能升级为实际结果。</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -19813,22 +19809,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I25" t="str">
-        <x:v>吨钢降本：原页面写为 63.7 元/吨。</x:v>
+        <x:v>2015年技术方案测算值：天然气117元/吨-冷煤气53.3元/吨=63.7元/吨燃料成本差额。</x:v>
       </x:c>
       <x:c r="J25" t="str">
-        <x:v>必须明确分母、成本项、含税口径、燃料结构、基准期与验证期，且只能适用于该项目。</x:v>
+        <x:v>分母为吨钢，分子只覆盖方案中的燃料成本差额；能源价格、热值、税口径和统计期决定结果。</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>复核单位产品成本计算、能源单价、产量分母和改造前后可比条件。</x:v>
+        <x:v>复核方案算术来源；后续仍需实际能源单价、热值、同工况吨钢能耗和完整统计期。</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>可公开为“单位产品能耗成本具备下降空间，幅度按现场数据单独核算”。</x:v>
+        <x:v>2015年技术方案按当时能源价格测算，单位吨钢燃料成本差额为63.7元；仅为本项目方案测算，不代表全部生产成本或实际验收结果。</x:v>
       </x:c>
       <x:c r="M25" t="str">
-        <x:v>唐工完成技术复核前，不公开 63.7 元/吨，不与任何未核年产量拼接成收益公式。</x:v>
+        <x:v>不得扩展成全部生产成本降幅；不得脱离能源价格和项目工况引用；唐工复核前不得跨页面或站外复用。</x:v>
       </x:c>
       <x:c r="N25" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>本项目技术方案“三、项目说明—A、经济性分析”：30Nm³/吨×3.9元/Nm³=117元/吨；标准煤暂估800元/吨，冷煤气折算53.3元/吨钢；差额63.7元/吨。未检出实际单位成本验证底稿。</x:v>
       </x:c>
       <x:c r="O25" t="str">
         <x:v>是</x:v>
@@ -19855,12 +19851,9 @@
       <x:c r="V25" t="str">
         <x:v>待安排：唐工</x:v>
       </x:c>
-      <x:c r="W25"/>
+      <x:c r="W25" s="30"/>
       <x:c r="X25" t="str">
-        <x:v>所需证据：吨产品成本计算底稿、能源单价、产量分母、统计期说明、技术审核、公司批准、客户授权。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：117、53.3和63.7的算术来源已找到；未检出实际单位成本验证底稿，方案也未明确含税口径、可比统计期及异常工况剔除规则。</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -19889,22 +19882,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I26" t="str">
-        <x:v>年产量/测算分母：原页面写为 120 万吨/年。</x:v>
+        <x:v>120万吨/年为2015年技术方案中三条线收益测算的年产量假设。</x:v>
       </x:c>
       <x:c r="J26" t="str">
-        <x:v>产能、实际产量与测算分母必须区分；该数据可能涉及客户经营信息。</x:v>
+        <x:v>该数用于经济性测算，当前证据不能证明其为客户实际有效产量、合格产量或经验证设计产能。</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>核对产量来源、统计口径及其是否仅为测算假设，确认客户允许公开的层级。</x:v>
+        <x:v>复核方案中的测算分母；后续仍需假设形成依据、实际生产台账和对应统计周期。</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>可公开为“收益测算需使用经双方确认的有效产量或运行负荷”。</x:v>
+        <x:v>2015年技术方案按三条线年产量120万吨进行收益测算；该数为方案假设，不代表客户实际年产量或经营结果。</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>唐工完成技术复核前，不公开 120 万吨/年，不将测算分母描述为客户实际产能或经营数据。</x:v>
+        <x:v>不得描述为客户实际有效产量、合格产量、实际经营数据或经验证设计产能；唐工复核前不得跨页面或站外复用。</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>本项目技术方案“三、项目说明—A、经济性分析”原文：“三条线按年产量120万吨计算”。该数是收益测算假设，未检出实际有效产量或合格产量台账。</x:v>
       </x:c>
       <x:c r="O26" t="str">
         <x:v>是</x:v>
@@ -19931,12 +19924,9 @@
       <x:c r="V26" t="str">
         <x:v>待安排：唐工</x:v>
       </x:c>
-      <x:c r="W26"/>
+      <x:c r="W26" s="30"/>
       <x:c r="X26" t="str">
-        <x:v>所需证据：产量台账或双方确认的测算假设、口径说明、公司批准、客户授权。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：技术方案直接写明“按年产量120万吨计算”，故可判定为三条线合计的收益测算假设；仍待唐工复核其形成依据和适用边界。</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -19965,22 +19955,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I27" t="str">
-        <x:v>项目周期：原页面写有 30-45 个工作日、4-6 个月、每条线 30-60 天等节点。</x:v>
+        <x:v>主合同节点：2015-11-15前具备安装条件，三条线分别于2015-12-05、2016-01-05、2016-02-05前完成；实施时间由买方安排。技术方案另载50个工作日、首线15～20日及每月一线的计划口径。</x:v>
       </x:c>
       <x:c r="J27" t="str">
-        <x:v>周期受停产窗口、供货边界、现场条件、材料交期和验收安排影响，只能按合同项目核实。</x:v>
+        <x:v>合同里程碑与技术方案计划必须分开；节点受现场条件、停产窗口、买方安排和不可抗力影响。</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>核对合同里程碑、生产排程、进场记录、调试与验收记录。</x:v>
+        <x:v>核对合同交货期与技术方案工期承诺；如需证明实际完成周期，另调进场、调试、烘炉和验收记录。</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>可公开为“各阶段周期按项目规模、供货边界和停产窗口在合同中确认”。</x:v>
+        <x:v>本项目合同约定分三条线实施并由买方按现场情况安排；各阶段周期以项目规模、供货边界、现场条件和停产窗口为准。</x:v>
       </x:c>
       <x:c r="M27" t="str">
-        <x:v>唐工完成技术复核且取得完整里程碑证据前，不公开固定设计、制造、安装或验收周期。</x:v>
+        <x:v>不得把本项目合同日期或技术方案计划改写成通用固定设计、制造、安装、停产或验收周期。</x:v>
       </x:c>
       <x:c r="N27" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>主合同第3页“四、交货期”：2015-11-15前具备安装条件，2015-12-05/2016-01-05/2016-02-05前分别完成三条线，具体实施时间由买方安排；技术方案5.1另载50个工作日、首线15～20日及每月一线的计划口径。</x:v>
       </x:c>
       <x:c r="O27" t="str">
         <x:v>是</x:v>
@@ -19992,7 +19982,7 @@
         <x:v>连续退洗线节能改造现有案例页</x:v>
       </x:c>
       <x:c r="R27" t="str">
-        <x:v>待唐工复核</x:v>
+        <x:v>资料确认</x:v>
       </x:c>
       <x:c r="S27" t="str">
         <x:v>通过</x:v>
@@ -20002,17 +19992,16 @@
       </x:c>
       <x:c r="U27" t="str">
         <x:f>IF(OR(R27="禁发",S27="禁发",T27="禁发"),"禁发",IF(AND(R27="资料确认",S27="通过",T27="通过"),"资料参数可发布",IF(AND(R27="行业推定",S27="通过",T27="通过"),"范围表达可发布",IF(AND(R27="通过",S27="通过",T27="通过"),"精确值可发布",IF(AND(S27="通过",R27="待唐工复核",T27="通过"),"公开（技术复核待完成）","待审核")))))</x:f>
-        <x:v>公开（技术复核待完成）</x:v>
+        <x:v>资料参数可发布</x:v>
       </x:c>
       <x:c r="V27" t="str">
-        <x:v>待安排：唐工</x:v>
-      </x:c>
-      <x:c r="W27"/>
+        <x:v>合同/技术方案资料核对</x:v>
+      </x:c>
+      <x:c r="W27" s="30" t="n">
+        <x:v>46234</x:v>
+      </x:c>
       <x:c r="X27" t="str">
-        <x:v>所需证据：合同计划、排产记录、进场/调试/验收日期、技术审核、公司批准、客户授权。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：合同第3页交货期为直接条款；技术方案5.1为计划口径。二者不得拼接。资料确认只证明约定节点，不证明实际完成日期。</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -20041,22 +20030,22 @@
         <x:v>改造</x:v>
       </x:c>
       <x:c r="I28" t="str">
-        <x:v>NOx 达标结论：原页面写为改造后满足 GB 28665-2012 及项目所在地环保要求。</x:v>
+        <x:v>技术方案采用低NOx烧嘴并作“改造后能够满足环保要求”的方案判断；本机未检出本项目第三方检测或正式验收报告。</x:v>
       </x:c>
       <x:c r="J28" t="str">
-        <x:v>排放结论必须对应适用标准、测试条件、检测机构、检测日期和具体项目边界。</x:v>
+        <x:v>二期其他生产线使用数据不能替代本项目检测结果；排放结论必须对应标准、工况、测点、检测机构和氧含量折算口径。</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>核对第三方检测或正式验收报告，并确认标准版本、限值、工况与测点。</x:v>
+        <x:v>调取本项目第三方检测或正式验收报告，并由唐工复核适用标准、测试条件和方案边界。</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>可公开为“按所在地排放要求设计，是否达标以有资质第三方检测或正式验收为准”。</x:v>
+        <x:v>按所在地排放要求设计，是否达标以有资质第三方检测或正式验收为准。</x:v>
       </x:c>
       <x:c r="M28" t="str">
-        <x:v>未取得可核验报告并完成唐工技术复核前，不写“已达标”“满足国家标准”或具体排放数值。</x:v>
+        <x:v>在取得可核验报告前，不写“已达标”“满足国家标准”或具体排放数值；不得用二期其他生产线数据替代一期检测结果。</x:v>
       </x:c>
       <x:c r="N28" t="str">
-        <x:v>现官网案例页待核事实；需回查合同、技术附件、计算底稿或验收资料</x:v>
+        <x:v>本项目技术方案“三、项目说明—B、满足环保性能要求”：采用低NOx烧嘴，并引用二期4#/5#线使用数据作方案判断。本机资料未检出本项目第三方检测或正式验收报告，需向公司/客户调取。</x:v>
       </x:c>
       <x:c r="O28" t="str">
         <x:v>是</x:v>
@@ -20083,12 +20072,9 @@
       <x:c r="V28" t="str">
         <x:v>待安排：唐工</x:v>
       </x:c>
-      <x:c r="W28"/>
+      <x:c r="W28" s="30"/>
       <x:c r="X28" t="str">
-        <x:v>所需证据：第三方检测/验收报告、适用标准与测试条件、技术审核、公司批准、客户授权。
-2026-07-29 授权确认：钱波确认台账当前表述均已获授权；授权范围限于本行已记录的公开或脱敏内容。
-GEO 决策：现有页面可按本行口径保留；唐工技术复核完成前，不新增未经复核的精确值，不跨页面复用，不站外分发。
-2026-07-29 发布决定：钱波完成行业常识初筛并确认当前内容上线；这不是唐工技术签审，公开时必须保留项目级适用边界。</x:v>
+        <x:v>2026-07-31 原件核查：仅找到技术方案中的设计/判断性表述；未检出检测机构、报告编号、检测日期、测点、工况、实测值、限值或氧含量折算口径。当前仅允许范围表达。</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -20573,7 +20559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R739ffce751c6460f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R089b408e847243f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>